<commit_message>
Add Fantom5, Vista and RefSeq CREs and related information
</commit_message>
<xml_diff>
--- a/data/files_provenance_ECCB-2026-T6.xlsx
+++ b/data/files_provenance_ECCB-2026-T6.xlsx
@@ -10,14 +10,14 @@
   <calcPr/>
   <extLst>
     <ext uri="GoogleSheetsCustomDataVersion2">
-      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId6" roundtripDataChecksum="H1VuZ+Wgg0UCk+fJGG0NY2lfCoooMpGuFz9Nr1Dtcdo="/>
+      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId6" roundtripDataChecksum="GKSCo0ojxI8ZjUlxdoIabpxHFONFuc30jw5nNNAgWGk="/>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="415" uniqueCount="128">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="446" uniqueCount="149">
   <si>
     <t>Folder</t>
   </si>
@@ -40,6 +40,9 @@
     <t>Version</t>
   </si>
   <si>
+    <t>Release</t>
+  </si>
+  <si>
     <t>Assembly</t>
   </si>
   <si>
@@ -49,64 +52,70 @@
     <t>Coordinate system</t>
   </si>
   <si>
-    <t>Release</t>
+    <t>Ensembl_Regulation</t>
   </si>
   <si>
     <t>ENCODE</t>
   </si>
   <si>
+    <t>GRCh38-cCRE-colors18062026.bed.gz</t>
+  </si>
+  <si>
+    <t>GRCh38-cCREs.bed</t>
+  </si>
+  <si>
     <t>ENCFF345CWR.atac.bed</t>
   </si>
   <si>
     <t>ENCFF345CWR.bed</t>
   </si>
   <si>
+    <t>ENCODE SCREEN</t>
+  </si>
+  <si>
+    <t>https://screen.wenglab.org/downloads</t>
+  </si>
+  <si>
+    <t>https://www.encodeproject.org/experiments/ENCSR903GMO/</t>
+  </si>
+  <si>
+    <t>V4</t>
+  </si>
+  <si>
+    <t>ENCODE4 v1.8.0</t>
+  </si>
+  <si>
+    <t>GRCh38</t>
+  </si>
+  <si>
+    <t>Added feature colors. Gzip compression</t>
+  </si>
+  <si>
+    <t>mm10</t>
+  </si>
+  <si>
+    <t>0-based</t>
+  </si>
+  <si>
+    <t>Rename to include assay type</t>
+  </si>
+  <si>
+    <t>ENCFF633ETU.atac.chr6.5911252-7710120.bw</t>
+  </si>
+  <si>
+    <t>ENCFF633ETU.bigWig</t>
+  </si>
+  <si>
+    <t>GRCh38-cCRE-colors18062026.bed.idx</t>
+  </si>
+  <si>
     <t>GRCh38-cCRE-colors18062026.bed</t>
   </si>
   <si>
-    <t>https://www.encodeproject.org/experiments/ENCSR903GMO/</t>
-  </si>
-  <si>
-    <t>GRCh38-cCREs.bed</t>
-  </si>
-  <si>
-    <t>ENCODE SCREEN</t>
-  </si>
-  <si>
-    <t>https://screen.wenglab.org/downloads</t>
-  </si>
-  <si>
-    <t>ENCODE4 v1.8.0</t>
-  </si>
-  <si>
-    <t>mm10</t>
-  </si>
-  <si>
-    <t>Rename to include assay type</t>
-  </si>
-  <si>
-    <t>0-based</t>
-  </si>
-  <si>
-    <t>V4</t>
-  </si>
-  <si>
-    <t>ENCFF633ETU.atac.chr6.5911252-7710120.bw</t>
-  </si>
-  <si>
-    <t>ENCFF633ETU.bigWig</t>
-  </si>
-  <si>
-    <t>GRCh38</t>
-  </si>
-  <si>
-    <t>Added feature colors</t>
-  </si>
-  <si>
     <t xml:space="preserve">Rename to include assay type. Trimming </t>
   </si>
   <si>
-    <t>GRCh38-cCRE-colors18062026.bed.idx</t>
+    <t>Bed file index</t>
   </si>
   <si>
     <t>ENCFF053ITU.k27ac.bed</t>
@@ -115,31 +124,31 @@
     <t>ENCFF053ITU.bed</t>
   </si>
   <si>
+    <t>GRCm39-cCRE-colors18062026.bed.gz</t>
+  </si>
+  <si>
+    <t>mm10-cCREs.bed</t>
+  </si>
+  <si>
     <t>https://www.encodeproject.org/experiments/ENCSR311YPF/</t>
   </si>
   <si>
+    <t>GRCm39</t>
+  </si>
+  <si>
     <t>ENCODE4 v1.5.1</t>
   </si>
   <si>
-    <t>Bed file index</t>
-  </si>
-  <si>
     <t>ENCFF607CHT.k27ac.chr6.5911252-7710120.bw</t>
   </si>
   <si>
-    <t>GRCm39-cCRE-colors18062026.bed</t>
-  </si>
-  <si>
     <t>ENCFF607CHT.bigWig</t>
   </si>
   <si>
-    <t>mm10-cCREs.bed</t>
-  </si>
-  <si>
-    <t>GRCm39</t>
-  </si>
-  <si>
-    <t>Liftover from mm10, add feature colors</t>
+    <t>Liftover from mm10, add feature colors. Gzip compression</t>
+  </si>
+  <si>
+    <t>mm10-cCRE-colors18062026.bed.gz</t>
   </si>
   <si>
     <t>ENCFF079TUC.k4me3.bed</t>
@@ -151,7 +160,10 @@
     <t>https://www.encodeproject.org/experiments/ENCSR835BZO/</t>
   </si>
   <si>
-    <t>mm10-cCRE-colors18062026.bed</t>
+    <t>HCT116-cCRE.chr8.bed</t>
+  </si>
+  <si>
+    <t>ENCFF431JDU_ENCFF964OOU_ENCFF787LMI_ENCFF388PVO.bed</t>
   </si>
   <si>
     <t>ENCFF798ETE.k4me3.chr6.5911252-7710120.bw</t>
@@ -160,37 +172,34 @@
     <t>ENCFF798ETE.bigWig</t>
   </si>
   <si>
-    <t>HCT116-cCRE.chr8.bed</t>
-  </si>
-  <si>
-    <t>ENCFF431JDU_ENCFF964OOU_ENCFF787LMI_ENCFF388PVO.bed</t>
+    <t>Filter chr8 features. Rename. Gzip compression.</t>
   </si>
   <si>
     <t>ENCFF217ZPW.k4me1.bed</t>
   </si>
   <si>
+    <t>Homo_sapiens.GRCh38.regulatory_features.v116.bb</t>
+  </si>
+  <si>
     <t>ENCFF217ZPW.bed</t>
   </si>
   <si>
-    <t>Filter chr8 features. Rename</t>
+    <t>Ensembl Regulation</t>
+  </si>
+  <si>
+    <t>https://regulation.ensembl.org/regulatory_features/homo_sapiens</t>
   </si>
   <si>
     <t>https://www.encodeproject.org/experiments/ENCSR496TBX/</t>
   </si>
   <si>
-    <t>Ensembl_Regulation</t>
-  </si>
-  <si>
-    <t>Homo_sapiens.GRCh38.regulatory_features.v116.bb</t>
+    <t>2025-12</t>
   </si>
   <si>
     <t>ENCODE4 v1.6.1</t>
   </si>
   <si>
-    <t>Ensembl Regulation</t>
-  </si>
-  <si>
-    <t>https://regulation.ensembl.org/regulatory_features/homo_sapiens</t>
+    <t>Homo_sapiens.GRCh38.regulatory_features.v116.gff3.gz</t>
   </si>
   <si>
     <t>ENCFF013ALT.k4me1.chr6.5911252-7710120.bw</t>
@@ -199,28 +208,28 @@
     <t>ENCFF013ALT.bigWig</t>
   </si>
   <si>
+    <t>1-based</t>
+  </si>
+  <si>
+    <t>Mus_musculus.GRCm39.regulatory_features.v116.bb</t>
+  </si>
+  <si>
     <t>ENCFF240LRP.dnase.bed</t>
   </si>
   <si>
-    <t>Homo_sapiens.GRCh38.regulatory_features.v116.gff3.gz</t>
-  </si>
-  <si>
     <t>ENCFF240LRP.bed</t>
   </si>
   <si>
+    <t>https://regulation.ensembl.org/regulatory_features/mus_musculus</t>
+  </si>
+  <si>
     <t>https://www.encodeproject.org/experiments/ENCSR000ENM/</t>
   </si>
   <si>
-    <t>1-based</t>
-  </si>
-  <si>
-    <t>Mus_musculus.GRCm39.regulatory_features.v116.bb</t>
-  </si>
-  <si>
     <t xml:space="preserve">ENCODE4 v3.0.0-alpha.2 </t>
   </si>
   <si>
-    <t>https://regulation.ensembl.org/regulatory_features/mus_musculus</t>
+    <t>Mus_musculus.GRCm39.regulatory_features.v116.gff3.gz</t>
   </si>
   <si>
     <t>ENCFF906MKW.dnase.chr8.126229903-128914986.bw</t>
@@ -229,27 +238,60 @@
     <t>ENCFF906MKW.bigWig</t>
   </si>
   <si>
-    <t>Mus_musculus.GRCm39.regulatory_features.v116.gff3.gz</t>
+    <t>Vista</t>
   </si>
   <si>
     <t>ENCFF296ZZB.atac.bed</t>
   </si>
   <si>
+    <t>vistaEnhancers_GRCh38.bb</t>
+  </si>
+  <si>
     <t>ENCFF296ZZB.bed</t>
   </si>
   <si>
+    <t>vistaEnhancers.bb</t>
+  </si>
+  <si>
     <t>https://www.encodeproject.org/experiments/ENCSR872WGW/</t>
   </si>
   <si>
+    <t>UCSC</t>
+  </si>
+  <si>
+    <t>https://hgdownload.soe.ucsc.edu/gbdb/hg38/vistaEnhancers/</t>
+  </si>
+  <si>
     <t>ENCODE4 v1.9.1</t>
   </si>
   <si>
+    <t>01/07/2026</t>
+  </si>
+  <si>
     <t>ENCFF624HRW.atac.chr8.126229903-128914986.bw</t>
   </si>
   <si>
     <t>ENCFF624HRW.bw</t>
   </si>
   <si>
+    <t>Rename</t>
+  </si>
+  <si>
+    <t>Fantom5</t>
+  </si>
+  <si>
+    <t>F5.hg38.enhancers.bed.gz</t>
+  </si>
+  <si>
+    <t>F5.hg38.enhancers.bed</t>
+  </si>
+  <si>
+    <t>Fantom</t>
+  </si>
+  <si>
+    <t>https://fantom.gsc.riken.jp/5/datafiles/reprocessed/hg38_v9/extra/enhancer/</t>
+  </si>
+  <si>
     <t>ENCFF711MPL.k4me3.bed</t>
   </si>
   <si>
@@ -259,15 +301,39 @@
     <t>https://www.encodeproject.org/experiments/ENCSR333OPW/</t>
   </si>
   <si>
+    <t>V9</t>
+  </si>
+  <si>
+    <t>Gzip compression.</t>
+  </si>
+  <si>
     <t xml:space="preserve">ENCODE4 v1.5.1 </t>
   </si>
   <si>
+    <t>RefSeq</t>
+  </si>
+  <si>
+    <t>GCF_000001405.40_GRCh38.p14_genomic.RefSeqFE.gff.gz</t>
+  </si>
+  <si>
+    <t>GCF_000001405.40_GRCh38.p14_genomic.gff</t>
+  </si>
+  <si>
     <t>ENCFF394IMO.k4me3.chr8.126229903-128914986.bw</t>
   </si>
   <si>
     <t>ENCFF394IMO.bw</t>
   </si>
   <si>
+    <t>https://ftp.ncbi.nlm.nih.gov/genomes/refseq/vertebrate_mammalian/Homo_sapiens/latest_assembly_versions/GCF_000001405.40_GRCh38.p14/</t>
+  </si>
+  <si>
+    <t>08/01/2025</t>
+  </si>
+  <si>
+    <t>Extract RefSeqFE annotations, rename chromosome, remove biological_region features. Gzip compression.</t>
+  </si>
+  <si>
     <t>ENCFF349LKU.k27ac.bed</t>
   </si>
   <si>
@@ -302,9 +368,6 @@
   </si>
   <si>
     <t>https://regulation.ensembl.org/epigenomes/mus_musculus/fW34w--4T_-CCG0vmtv3bQ</t>
-  </si>
-  <si>
-    <t>2025-12</t>
   </si>
   <si>
     <t>atac_seq_forebrain_m_13.5_d.bed.gz</t>
@@ -407,11 +470,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <numFmts count="2">
+  <numFmts count="1">
     <numFmt numFmtId="164" formatCode="dd/mm/yyyy"/>
-    <numFmt numFmtId="165" formatCode="yyyy-m"/>
   </numFmts>
-  <fonts count="14">
+  <fonts count="16">
     <font>
       <sz val="10.0"/>
       <color rgb="FF000000"/>
@@ -447,6 +509,21 @@
     </font>
     <font>
       <u/>
+      <color rgb="FF0000FF"/>
+      <name val="Roboto"/>
+    </font>
+    <font>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
       <color rgb="FF434343"/>
       <name val="Roboto"/>
     </font>
@@ -466,11 +543,6 @@
     <font>
       <color rgb="FF000000"/>
       <name val="Roboto"/>
-    </font>
-    <font>
-      <color theme="1"/>
-      <name val="Arial"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <u/>
@@ -546,12 +618,18 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="46">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="center" wrapText="0"/>
@@ -566,19 +644,19 @@
       <alignment shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
     <xf borderId="0" fillId="2" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
-      <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="0"/>
+      <alignment shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="165" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="0"/>
+    <xf borderId="0" fillId="0" fontId="1" numFmtId="49" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+      <alignment shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
@@ -586,46 +664,76 @@
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="49" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
-      <alignment shrinkToFit="0" vertical="center" wrapText="0"/>
-    </xf>
-    <xf borderId="1" fillId="2" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment shrinkToFit="0" vertical="center" wrapText="0"/>
-    </xf>
-    <xf borderId="2" fillId="2" fontId="8" numFmtId="164" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="right" shrinkToFit="0" vertical="center" wrapText="0"/>
-    </xf>
-    <xf borderId="2" fillId="2" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment shrinkToFit="0" vertical="center" wrapText="0"/>
-    </xf>
-    <xf borderId="2" fillId="2" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment shrinkToFit="0" vertical="center" wrapText="0"/>
-    </xf>
-    <xf borderId="2" fillId="2" fontId="8" numFmtId="49" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
-      <alignment shrinkToFit="0" vertical="center" wrapText="0"/>
-    </xf>
-    <xf borderId="2" fillId="2" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment shrinkToFit="0" vertical="center" wrapText="0"/>
-    </xf>
-    <xf borderId="3" fillId="2" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment shrinkToFit="0" vertical="center" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
+    <xf borderId="0" fillId="0" fontId="1" numFmtId="164" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="1" numFmtId="49" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="8" numFmtId="49" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
+    </xf>
     <xf borderId="0" fillId="0" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="12" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="1" fillId="2" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment shrinkToFit="0" vertical="center" wrapText="0"/>
+    </xf>
+    <xf borderId="2" fillId="2" fontId="11" numFmtId="164" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="right" shrinkToFit="0" vertical="center" wrapText="0"/>
+    </xf>
+    <xf borderId="2" fillId="2" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment shrinkToFit="0" vertical="center" wrapText="0"/>
+    </xf>
+    <xf borderId="2" fillId="2" fontId="12" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment shrinkToFit="0" vertical="center" wrapText="0"/>
+    </xf>
+    <xf borderId="2" fillId="2" fontId="11" numFmtId="49" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+      <alignment shrinkToFit="0" vertical="center" wrapText="0"/>
+    </xf>
+    <xf borderId="2" fillId="2" fontId="13" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment shrinkToFit="0" vertical="center" wrapText="0"/>
+    </xf>
+    <xf borderId="3" fillId="2" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment shrinkToFit="0" vertical="center" wrapText="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="14" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="13" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="14" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
     <xf borderId="1" fillId="3" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
@@ -637,13 +745,13 @@
     <xf borderId="2" fillId="3" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
-    <xf borderId="2" fillId="3" fontId="13" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="2" fillId="3" fontId="15" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
     <xf borderId="2" fillId="3" fontId="1" numFmtId="49" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
-    <xf borderId="2" fillId="3" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="2" fillId="3" fontId="13" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
     <xf borderId="3" fillId="3" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
@@ -709,13 +817,13 @@
     </dxf>
   </dxfs>
   <tableStyles count="2">
-    <tableStyle count="4" pivot="0" name="Evidence-style">
+    <tableStyle count="4" pivot="0" name="CREs annotation-style">
       <tableStyleElement dxfId="1" type="headerRow"/>
       <tableStyleElement dxfId="2" type="firstRowStripe"/>
       <tableStyleElement dxfId="3" type="secondRowStripe"/>
       <tableStyleElement dxfId="4" size="0" type="wholeTable"/>
     </tableStyle>
-    <tableStyle count="4" pivot="0" name="CREs annotation-style">
+    <tableStyle count="4" pivot="0" name="Evidence-style">
       <tableStyleElement dxfId="1" type="headerRow"/>
       <tableStyleElement dxfId="2" type="firstRowStripe"/>
       <tableStyleElement dxfId="3" type="secondRowStripe"/>
@@ -734,7 +842,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:J10" displayName="Table2" name="Table2" id="2">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:J13" displayName="Table2" name="Table2" id="2">
   <tableColumns count="10">
     <tableColumn name="Folder" id="1"/>
     <tableColumn name="File name" id="2"/>
@@ -970,12 +1078,13 @@
   </sheetPr>
   <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.0"/>
   <cols>
-    <col customWidth="1" min="1" max="1" width="28.5"/>
-    <col customWidth="1" min="2" max="3" width="37.63"/>
+    <col customWidth="1" min="1" max="1" width="18.88"/>
+    <col customWidth="1" min="2" max="2" width="45.25"/>
+    <col customWidth="1" min="3" max="3" width="37.63"/>
     <col customWidth="1" min="4" max="4" width="19.88"/>
     <col customWidth="1" min="5" max="5" width="21.0"/>
     <col customWidth="1" min="6" max="6" width="37.63"/>
-    <col customWidth="1" min="7" max="7" width="11.38"/>
+    <col customWidth="1" min="7" max="7" width="16.25"/>
     <col customWidth="1" min="8" max="8" width="12.75"/>
     <col customWidth="1" min="9" max="9" width="31.25"/>
     <col customWidth="1" min="10" max="10" width="22.75"/>
@@ -1001,291 +1110,384 @@
         <v>5</v>
       </c>
       <c r="G1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="J1" s="1" t="s">
         <v>10</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>9</v>
       </c>
     </row>
     <row r="2" ht="22.5" customHeight="1">
       <c r="A2" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C2" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="C2" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="D2" s="3">
+      <c r="D2" s="5">
         <v>46191.0</v>
       </c>
-      <c r="E2" s="4" t="s">
+      <c r="E2" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="F2" s="5" t="s">
+      <c r="F2" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="G2" s="6" t="s">
+      <c r="G2" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="H2" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="I2" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="H2" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="I2" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="J2" s="4" t="s">
+      <c r="J2" s="6" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="3" ht="22.5" customHeight="1">
+      <c r="A3" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="D3" s="5"/>
+      <c r="E3" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="F3" s="10"/>
+      <c r="G3" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="H3" s="9" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="3" ht="22.5" customHeight="1">
-      <c r="A3" s="7" t="s">
+      <c r="I3" s="9" t="s">
+        <v>32</v>
+      </c>
+      <c r="J3" s="6"/>
+    </row>
+    <row r="4" ht="22.5" customHeight="1">
+      <c r="A4" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="D4" s="5">
+        <v>46191.0</v>
+      </c>
+      <c r="E4" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="F4" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="G4" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="H4" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="I4" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="J4" s="6" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="5" ht="22.5" customHeight="1">
+      <c r="A5" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="D5" s="5">
+        <v>46191.0</v>
+      </c>
+      <c r="E5" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="F5" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="G5" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="H5" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="I5" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="J5" s="6" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="6" ht="22.5" customHeight="1">
+      <c r="A6" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="D6" s="5">
+        <v>46227.0</v>
+      </c>
+      <c r="E6" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="F6" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="G6" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="H6" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="I6" s="9" t="s">
+        <v>51</v>
+      </c>
+      <c r="J6" s="6" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="7" ht="22.5" customHeight="1">
+      <c r="A7" s="11" t="s">
         <v>11</v>
       </c>
-      <c r="B3" s="7" t="s">
-        <v>29</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="D3" s="3"/>
-      <c r="E3" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="F3" s="8"/>
-      <c r="G3" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="H3" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="I3" s="9" t="s">
-        <v>34</v>
-      </c>
-      <c r="J3" s="4"/>
-    </row>
-    <row r="4" ht="22.5" customHeight="1">
-      <c r="A4" s="2" t="s">
+      <c r="B7" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="D7" s="5">
+        <v>46206.0</v>
+      </c>
+      <c r="E7" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="F7" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="G7" s="12" t="s">
+        <v>58</v>
+      </c>
+      <c r="H7" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="J7" s="6" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="8" ht="22.5" customHeight="1">
+      <c r="A8" s="11" t="s">
         <v>11</v>
       </c>
-      <c r="B4" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="C4" s="2" t="s">
+      <c r="B8" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="D8" s="5">
+        <v>46191.0</v>
+      </c>
+      <c r="E8" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="F8" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="G8" s="12" t="s">
+        <v>58</v>
+      </c>
+      <c r="H8" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="J8" s="6" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="9" ht="22.5" customHeight="1">
+      <c r="A9" s="11" t="s">
+        <v>11</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="D9" s="5">
+        <v>46206.0</v>
+      </c>
+      <c r="E9" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="F9" s="13" t="s">
+        <v>67</v>
+      </c>
+      <c r="G9" s="12" t="s">
+        <v>58</v>
+      </c>
+      <c r="H9" s="6" t="s">
         <v>38</v>
       </c>
-      <c r="D4" s="3">
+      <c r="J9" s="6" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="10" ht="22.5" customHeight="1">
+      <c r="A10" s="11" t="s">
+        <v>11</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>70</v>
+      </c>
+      <c r="C10" s="4" t="s">
+        <v>70</v>
+      </c>
+      <c r="D10" s="5">
         <v>46191.0</v>
       </c>
-      <c r="E4" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="F4" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="G4" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="H4" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="I4" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="J4" s="4" t="s">
+      <c r="E10" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="F10" s="13" t="s">
+        <v>67</v>
+      </c>
+      <c r="G10" s="12" t="s">
+        <v>58</v>
+      </c>
+      <c r="H10" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="J10" s="6" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="11" ht="15.75" customHeight="1">
+      <c r="A11" s="14" t="s">
+        <v>73</v>
+      </c>
+      <c r="B11" s="15" t="s">
+        <v>75</v>
+      </c>
+      <c r="C11" s="16" t="s">
+        <v>77</v>
+      </c>
+      <c r="D11" s="17">
+        <v>46251.0</v>
+      </c>
+      <c r="E11" s="18" t="s">
+        <v>79</v>
+      </c>
+      <c r="F11" s="19" t="s">
+        <v>80</v>
+      </c>
+      <c r="G11" s="20" t="s">
+        <v>82</v>
+      </c>
+      <c r="H11" s="21" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="5" ht="22.5" customHeight="1">
-      <c r="A5" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>44</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="D5" s="3">
-        <v>46191.0</v>
-      </c>
-      <c r="E5" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="F5" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="G5" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="H5" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="I5" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="J5" s="4" t="s">
+      <c r="I11" s="22" t="s">
+        <v>85</v>
+      </c>
+      <c r="J11" s="6" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="12" ht="15.75" customHeight="1">
+      <c r="A12" s="14" t="s">
+        <v>86</v>
+      </c>
+      <c r="B12" s="23" t="s">
+        <v>87</v>
+      </c>
+      <c r="C12" s="23" t="s">
+        <v>88</v>
+      </c>
+      <c r="D12" s="17">
+        <v>46251.0</v>
+      </c>
+      <c r="E12" s="18" t="s">
+        <v>89</v>
+      </c>
+      <c r="F12" s="19" t="s">
+        <v>90</v>
+      </c>
+      <c r="G12" s="24" t="s">
+        <v>94</v>
+      </c>
+      <c r="H12" s="21" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="6" ht="22.5" customHeight="1">
-      <c r="A6" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="D6" s="3">
-        <v>46227.0</v>
-      </c>
-      <c r="E6" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="F6" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="G6" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="H6" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="I6" s="4" t="s">
-        <v>51</v>
-      </c>
-      <c r="J6" s="4" t="s">
+      <c r="I12" s="23" t="s">
+        <v>95</v>
+      </c>
+      <c r="J12" s="6" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="13" ht="15.75" customHeight="1">
+      <c r="A13" s="14" t="s">
+        <v>97</v>
+      </c>
+      <c r="B13" s="23" t="s">
+        <v>98</v>
+      </c>
+      <c r="C13" s="23" t="s">
+        <v>99</v>
+      </c>
+      <c r="D13" s="17">
+        <v>46251.0</v>
+      </c>
+      <c r="E13" s="18" t="s">
+        <v>97</v>
+      </c>
+      <c r="F13" s="19" t="s">
+        <v>102</v>
+      </c>
+      <c r="G13" s="20" t="s">
+        <v>103</v>
+      </c>
+      <c r="H13" s="21" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="7" ht="22.5" customHeight="1">
-      <c r="A7" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="D7" s="3">
-        <v>46206.0</v>
-      </c>
-      <c r="E7" s="4" t="s">
-        <v>56</v>
-      </c>
-      <c r="F7" s="5" t="s">
-        <v>57</v>
-      </c>
-      <c r="G7" s="10">
-        <v>45992.0</v>
-      </c>
-      <c r="H7" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="J7" s="4" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="8" ht="22.5" customHeight="1">
-      <c r="A8" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="C8" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="D8" s="3">
-        <v>46191.0</v>
-      </c>
-      <c r="E8" s="4" t="s">
-        <v>56</v>
-      </c>
-      <c r="F8" s="5" t="s">
-        <v>57</v>
-      </c>
-      <c r="G8" s="10">
-        <v>45992.0</v>
-      </c>
-      <c r="H8" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="J8" s="4" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="9" ht="22.5" customHeight="1">
-      <c r="A9" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="B9" s="2" t="s">
-        <v>65</v>
-      </c>
-      <c r="C9" s="2" t="s">
-        <v>65</v>
-      </c>
-      <c r="D9" s="3">
-        <v>46206.0</v>
-      </c>
-      <c r="E9" s="4" t="s">
-        <v>56</v>
-      </c>
-      <c r="F9" s="11" t="s">
-        <v>67</v>
-      </c>
-      <c r="G9" s="10">
-        <v>45992.0</v>
-      </c>
-      <c r="H9" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="J9" s="4" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="10" ht="22.5" customHeight="1">
-      <c r="A10" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="B10" s="2" t="s">
-        <v>70</v>
-      </c>
-      <c r="C10" s="2" t="s">
-        <v>70</v>
-      </c>
-      <c r="D10" s="3">
-        <v>46191.0</v>
-      </c>
-      <c r="E10" s="4" t="s">
-        <v>56</v>
-      </c>
-      <c r="F10" s="11" t="s">
-        <v>67</v>
-      </c>
-      <c r="G10" s="10">
-        <v>45992.0</v>
-      </c>
-      <c r="H10" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="J10" s="4" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="11" ht="15.75" customHeight="1"/>
-    <row r="12" ht="15.75" customHeight="1"/>
-    <row r="13" ht="15.75" customHeight="1"/>
+      <c r="I13" s="22" t="s">
+        <v>104</v>
+      </c>
+      <c r="J13" s="21" t="s">
+        <v>63</v>
+      </c>
+    </row>
     <row r="14" ht="15.75" customHeight="1"/>
     <row r="15" ht="15.75" customHeight="1"/>
     <row r="16" ht="15.75" customHeight="1"/>
@@ -2276,18 +2478,16 @@
     <row r="1001" ht="15.75" customHeight="1"/>
   </sheetData>
   <dataValidations>
-    <dataValidation type="custom" allowBlank="1" showDropDown="1" sqref="D2:D10">
+    <dataValidation type="list" allowBlank="1" sqref="A2:A13">
+      <formula1>"ENCODE,Ensembl_Regulation,Vista,Fantom5,RefSeq"</formula1>
+    </dataValidation>
+    <dataValidation type="custom" allowBlank="1" showDropDown="1" sqref="D2:D13">
       <formula1>OR(NOT(ISERROR(DATEVALUE(D2))), AND(ISNUMBER(D2), LEFT(CELL("format", D2))="D"))</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="A2:A10">
-      <formula1>"ENCODE,Ensembl_Regulation"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showDropDown="1" showErrorMessage="1" sqref="J2:J10">
+    <dataValidation type="list" allowBlank="1" showDropDown="1" showErrorMessage="1" sqref="J2:J13">
       <formula1>"0-based,1-based"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showDropDown="1" showErrorMessage="1" sqref="E2:E10">
-      <formula1>"ENCODE SCREEN,Ensembl Regulation"</formula1>
-    </dataValidation>
+    <dataValidation allowBlank="1" showDropDown="1" sqref="E2:E13 G2:G13"/>
   </dataValidations>
   <hyperlinks>
     <hyperlink r:id="rId1" ref="F2"/>
@@ -2298,10 +2498,13 @@
     <hyperlink r:id="rId6" ref="F8"/>
     <hyperlink r:id="rId7" ref="F9"/>
     <hyperlink r:id="rId8" ref="F10"/>
+    <hyperlink r:id="rId9" ref="F11"/>
+    <hyperlink r:id="rId10" ref="F12"/>
+    <hyperlink r:id="rId11" ref="F13"/>
   </hyperlinks>
-  <drawing r:id="rId9"/>
+  <drawing r:id="rId12"/>
   <tableParts count="1">
-    <tablePart r:id="rId11"/>
+    <tablePart r:id="rId14"/>
   </tableParts>
 </worksheet>
 </file>
@@ -2348,1180 +2551,1180 @@
         <v>6</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="2" ht="22.5" customHeight="1">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="D2" s="5">
+        <v>46226.0</v>
+      </c>
+      <c r="E2" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="F2" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="G2" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="H2" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="I2" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="J2" s="6" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="3" ht="22.5" customHeight="1">
+      <c r="A3" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="D3" s="5">
+        <v>46226.0</v>
+      </c>
+      <c r="E3" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="F3" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="G3" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="H3" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="I3" s="6" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="4" ht="22.5" customHeight="1">
+      <c r="A4" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="D4" s="5">
+        <v>46226.0</v>
+      </c>
+      <c r="E4" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="F4" s="7" t="s">
+        <v>37</v>
+      </c>
+      <c r="G4" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="H4" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="I4" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="J4" s="6" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="5" ht="22.5" customHeight="1">
+      <c r="A5" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="D5" s="5">
+        <v>46226.0</v>
+      </c>
+      <c r="E5" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="F5" s="7" t="s">
+        <v>37</v>
+      </c>
+      <c r="G5" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="H5" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="I5" s="6" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="6" ht="22.5" customHeight="1">
+      <c r="A6" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="D6" s="5">
+        <v>46226.0</v>
+      </c>
+      <c r="E6" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="F6" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="G6" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="H6" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="I6" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="J6" s="6" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="7" ht="22.5" customHeight="1">
+      <c r="A7" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="D7" s="5">
+        <v>46226.0</v>
+      </c>
+      <c r="E7" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="F7" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="G7" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="H7" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="I7" s="6" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="8" ht="22.5" customHeight="1">
+      <c r="A8" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="D8" s="5">
+        <v>46226.0</v>
+      </c>
+      <c r="E8" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="F8" s="7" t="s">
+        <v>57</v>
+      </c>
+      <c r="G8" s="6" t="s">
+        <v>59</v>
+      </c>
+      <c r="H8" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="I8" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="J8" s="6" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="9" ht="22.5" customHeight="1">
+      <c r="A9" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="D9" s="5">
+        <v>46226.0</v>
+      </c>
+      <c r="E9" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="F9" s="7" t="s">
+        <v>57</v>
+      </c>
+      <c r="G9" s="6" t="s">
+        <v>59</v>
+      </c>
+      <c r="H9" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="I9" s="6" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="10" ht="22.5" customHeight="1">
+      <c r="A10" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="C10" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="D10" s="5">
+        <v>46162.0</v>
+      </c>
+      <c r="E10" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="F10" s="7" t="s">
+        <v>68</v>
+      </c>
+      <c r="G10" s="6" t="s">
+        <v>69</v>
+      </c>
+      <c r="H10" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="I10" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="J10" s="6" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="11" ht="22.5" customHeight="1">
+      <c r="A11" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>71</v>
+      </c>
+      <c r="C11" s="4" t="s">
+        <v>72</v>
+      </c>
+      <c r="D11" s="5">
+        <v>46162.0</v>
+      </c>
+      <c r="E11" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="F11" s="7" t="s">
+        <v>68</v>
+      </c>
+      <c r="G11" s="6" t="s">
+        <v>69</v>
+      </c>
+      <c r="H11" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="I11" s="6" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="12" ht="22.5" customHeight="1">
+      <c r="A12" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="C12" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="D12" s="5">
+        <v>46162.0</v>
+      </c>
+      <c r="E12" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="F12" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="G12" s="6" t="s">
+        <v>81</v>
+      </c>
+      <c r="H12" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="I12" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="J12" s="6" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="13" ht="22.5" customHeight="1">
+      <c r="A13" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>83</v>
+      </c>
+      <c r="C13" s="6" t="s">
+        <v>84</v>
+      </c>
+      <c r="D13" s="5">
+        <v>46162.0</v>
+      </c>
+      <c r="E13" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="F13" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="G13" s="6" t="s">
+        <v>81</v>
+      </c>
+      <c r="H13" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="I13" s="6" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="14" ht="22.5" customHeight="1">
+      <c r="A14" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B14" s="4" t="s">
+        <v>91</v>
+      </c>
+      <c r="C14" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="D14" s="5">
+        <v>46162.0</v>
+      </c>
+      <c r="E14" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="F14" s="7" t="s">
+        <v>93</v>
+      </c>
+      <c r="G14" s="6" t="s">
+        <v>96</v>
+      </c>
+      <c r="H14" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="I14" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="J14" s="6" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="15" ht="22.5" customHeight="1">
+      <c r="A15" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B15" s="4" t="s">
+        <v>100</v>
+      </c>
+      <c r="C15" s="6" t="s">
+        <v>101</v>
+      </c>
+      <c r="D15" s="5">
+        <v>46162.0</v>
+      </c>
+      <c r="E15" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="F15" s="7" t="s">
+        <v>93</v>
+      </c>
+      <c r="G15" s="6" t="s">
+        <v>96</v>
+      </c>
+      <c r="H15" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="I15" s="6" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="16" ht="22.5" customHeight="1">
+      <c r="A16" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B16" s="4" t="s">
+        <v>105</v>
+      </c>
+      <c r="C16" s="4" t="s">
+        <v>106</v>
+      </c>
+      <c r="D16" s="5">
+        <v>46162.0</v>
+      </c>
+      <c r="E16" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="F16" s="7" t="s">
+        <v>107</v>
+      </c>
+      <c r="G16" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="H16" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="I16" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="J16" s="6" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="17" ht="22.5" customHeight="1">
+      <c r="A17" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B17" s="4" t="s">
+        <v>108</v>
+      </c>
+      <c r="C17" s="4" t="s">
+        <v>109</v>
+      </c>
+      <c r="D17" s="5">
+        <v>46162.0</v>
+      </c>
+      <c r="E17" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="F17" s="7" t="s">
+        <v>107</v>
+      </c>
+      <c r="G17" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="H17" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="I17" s="6" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="18" ht="22.5" customHeight="1">
+      <c r="A18" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B18" s="4" t="s">
+        <v>110</v>
+      </c>
+      <c r="C18" s="4" t="s">
+        <v>111</v>
+      </c>
+      <c r="D18" s="5">
+        <v>46162.0</v>
+      </c>
+      <c r="E18" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="F18" s="7" t="s">
+        <v>112</v>
+      </c>
+      <c r="G18" s="6" t="s">
+        <v>59</v>
+      </c>
+      <c r="H18" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="I18" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="J18" s="6" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="19" ht="22.5" customHeight="1">
+      <c r="A19" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B19" s="4" t="s">
+        <v>113</v>
+      </c>
+      <c r="C19" s="6" t="s">
+        <v>114</v>
+      </c>
+      <c r="D19" s="5">
+        <v>46162.0</v>
+      </c>
+      <c r="E19" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="F19" s="7" t="s">
+        <v>112</v>
+      </c>
+      <c r="G19" s="6" t="s">
+        <v>59</v>
+      </c>
+      <c r="H19" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="I19" s="6" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="20" ht="22.5" customHeight="1">
+      <c r="A20" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="B2" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="D2" s="3">
-        <v>46226.0</v>
-      </c>
-      <c r="E2" s="4" t="s">
+      <c r="B20" s="25" t="s">
+        <v>115</v>
+      </c>
+      <c r="C20" s="25" t="s">
+        <v>115</v>
+      </c>
+      <c r="D20" s="5">
+        <v>46227.0</v>
+      </c>
+      <c r="E20" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="F20" s="26" t="s">
+        <v>116</v>
+      </c>
+      <c r="G20" s="12" t="s">
+        <v>58</v>
+      </c>
+      <c r="H20" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="J20" s="6" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="21" ht="22.5" customHeight="1">
+      <c r="A21" s="27" t="s">
         <v>11</v>
       </c>
-      <c r="F2" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="G2" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="H2" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="I2" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="J2" s="4" t="s">
+      <c r="B21" s="3" t="s">
+        <v>117</v>
+      </c>
+      <c r="C21" s="25" t="s">
+        <v>115</v>
+      </c>
+      <c r="D21" s="28">
+        <v>46227.0</v>
+      </c>
+      <c r="E21" s="29" t="s">
+        <v>55</v>
+      </c>
+      <c r="F21" s="30" t="s">
+        <v>118</v>
+      </c>
+      <c r="G21" s="31" t="s">
+        <v>58</v>
+      </c>
+      <c r="H21" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="I21" s="32" t="s">
+        <v>119</v>
+      </c>
+      <c r="J21" s="33" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="22" ht="22.5" customHeight="1">
+      <c r="A22" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="B22" s="34" t="s">
+        <v>120</v>
+      </c>
+      <c r="C22" s="34" t="s">
+        <v>121</v>
+      </c>
+      <c r="D22" s="5">
+        <v>46227.0</v>
+      </c>
+      <c r="E22" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="F22" s="7" t="s">
+        <v>116</v>
+      </c>
+      <c r="G22" s="12" t="s">
+        <v>58</v>
+      </c>
+      <c r="H22" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="I22" s="6" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="23" ht="22.5" customHeight="1">
+      <c r="A23" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="B23" s="25" t="s">
+        <v>123</v>
+      </c>
+      <c r="C23" s="25" t="s">
+        <v>123</v>
+      </c>
+      <c r="D23" s="5">
+        <v>46227.0</v>
+      </c>
+      <c r="E23" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="F23" s="7" t="s">
+        <v>116</v>
+      </c>
+      <c r="G23" s="12" t="s">
+        <v>58</v>
+      </c>
+      <c r="H23" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="J23" s="6" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="24" ht="22.5" customHeight="1">
+      <c r="A24" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="B24" s="34" t="s">
+        <v>124</v>
+      </c>
+      <c r="C24" s="34" t="s">
+        <v>125</v>
+      </c>
+      <c r="D24" s="5">
+        <v>46227.0</v>
+      </c>
+      <c r="E24" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="F24" s="7" t="s">
+        <v>116</v>
+      </c>
+      <c r="G24" s="12" t="s">
+        <v>58</v>
+      </c>
+      <c r="H24" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="I24" s="6" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="25" ht="22.5" customHeight="1">
+      <c r="A25" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="B25" s="25" t="s">
+        <v>126</v>
+      </c>
+      <c r="C25" s="35" t="s">
+        <v>126</v>
+      </c>
+      <c r="D25" s="5">
+        <v>46227.0</v>
+      </c>
+      <c r="E25" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="F25" s="7" t="s">
+        <v>116</v>
+      </c>
+      <c r="G25" s="12" t="s">
+        <v>58</v>
+      </c>
+      <c r="H25" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="J25" s="6" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="26" ht="22.5" customHeight="1">
+      <c r="A26" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="B26" s="36" t="s">
+        <v>127</v>
+      </c>
+      <c r="C26" s="36" t="s">
+        <v>128</v>
+      </c>
+      <c r="D26" s="5">
+        <v>46227.0</v>
+      </c>
+      <c r="E26" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="F26" s="7" t="s">
+        <v>116</v>
+      </c>
+      <c r="G26" s="12" t="s">
+        <v>58</v>
+      </c>
+      <c r="H26" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="I26" s="6" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="27" ht="22.5" customHeight="1">
+      <c r="A27" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="B27" s="25" t="s">
+        <v>129</v>
+      </c>
+      <c r="C27" s="25" t="s">
+        <v>129</v>
+      </c>
+      <c r="D27" s="5">
+        <v>46227.0</v>
+      </c>
+      <c r="E27" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="F27" s="7" t="s">
+        <v>116</v>
+      </c>
+      <c r="G27" s="12" t="s">
+        <v>58</v>
+      </c>
+      <c r="H27" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="J27" s="6" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="28" ht="22.5" customHeight="1">
+      <c r="A28" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="B28" s="25" t="s">
+        <v>130</v>
+      </c>
+      <c r="C28" s="25" t="s">
+        <v>131</v>
+      </c>
+      <c r="D28" s="5">
+        <v>46227.0</v>
+      </c>
+      <c r="E28" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="F28" s="7" t="s">
+        <v>116</v>
+      </c>
+      <c r="G28" s="12" t="s">
+        <v>58</v>
+      </c>
+      <c r="H28" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="I28" s="6" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="29" ht="22.5" customHeight="1">
+      <c r="A29" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="B29" s="4" t="s">
+        <v>132</v>
+      </c>
+      <c r="C29" s="4" t="s">
+        <v>132</v>
+      </c>
+      <c r="D29" s="5">
+        <v>46227.0</v>
+      </c>
+      <c r="E29" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="F29" s="7" t="s">
+        <v>118</v>
+      </c>
+      <c r="G29" s="12" t="s">
+        <v>58</v>
+      </c>
+      <c r="H29" s="6" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="3" ht="22.5" customHeight="1">
-      <c r="A3" s="2" t="s">
+      <c r="J29" s="6" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="30" ht="22.5" customHeight="1">
+      <c r="A30" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="B3" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="C3" s="2" t="s">
+      <c r="B30" s="3" t="s">
+        <v>133</v>
+      </c>
+      <c r="C30" s="4" t="s">
+        <v>132</v>
+      </c>
+      <c r="D30" s="5">
+        <v>46227.0</v>
+      </c>
+      <c r="E30" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="F30" s="7" t="s">
+        <v>118</v>
+      </c>
+      <c r="G30" s="12" t="s">
+        <v>58</v>
+      </c>
+      <c r="H30" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="I30" s="37" t="s">
+        <v>119</v>
+      </c>
+      <c r="J30" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="D3" s="3">
-        <v>46226.0</v>
-      </c>
-      <c r="E3" s="4" t="s">
+    </row>
+    <row r="31" ht="22.5" customHeight="1">
+      <c r="A31" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="F3" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="G3" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="H3" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="I3" s="4" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="4" ht="22.5" customHeight="1">
-      <c r="A4" s="2" t="s">
+      <c r="B31" s="4" t="s">
+        <v>134</v>
+      </c>
+      <c r="C31" s="38" t="s">
+        <v>135</v>
+      </c>
+      <c r="D31" s="5">
+        <v>46227.0</v>
+      </c>
+      <c r="E31" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="F31" s="7" t="s">
+        <v>118</v>
+      </c>
+      <c r="G31" s="12" t="s">
+        <v>58</v>
+      </c>
+      <c r="H31" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="I31" s="6" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="32" ht="22.5" customHeight="1">
+      <c r="A32" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="B4" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="D4" s="3">
-        <v>46226.0</v>
-      </c>
-      <c r="E4" s="4" t="s">
+      <c r="B32" s="4" t="s">
+        <v>136</v>
+      </c>
+      <c r="C32" s="4" t="s">
+        <v>136</v>
+      </c>
+      <c r="D32" s="5">
+        <v>46227.0</v>
+      </c>
+      <c r="E32" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="F32" s="7" t="s">
+        <v>118</v>
+      </c>
+      <c r="G32" s="12" t="s">
+        <v>58</v>
+      </c>
+      <c r="H32" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="J32" s="6" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="33" ht="22.5" customHeight="1">
+      <c r="A33" s="39" t="s">
         <v>11</v>
       </c>
-      <c r="F4" s="5" t="s">
-        <v>32</v>
-      </c>
-      <c r="G4" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="H4" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="I4" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="J4" s="4" t="s">
+      <c r="B33" s="3" t="s">
+        <v>137</v>
+      </c>
+      <c r="C33" s="4" t="s">
+        <v>136</v>
+      </c>
+      <c r="D33" s="40">
+        <v>46227.0</v>
+      </c>
+      <c r="E33" s="41" t="s">
+        <v>55</v>
+      </c>
+      <c r="F33" s="42" t="s">
+        <v>118</v>
+      </c>
+      <c r="G33" s="43" t="s">
+        <v>58</v>
+      </c>
+      <c r="H33" s="41" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="5" ht="22.5" customHeight="1">
-      <c r="A5" s="2" t="s">
+      <c r="I33" s="44" t="s">
+        <v>119</v>
+      </c>
+      <c r="J33" s="45" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="34" ht="22.5" customHeight="1">
+      <c r="A34" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="B5" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="D5" s="3">
-        <v>46226.0</v>
-      </c>
-      <c r="E5" s="4" t="s">
+      <c r="B34" s="4" t="s">
+        <v>138</v>
+      </c>
+      <c r="C34" s="6" t="s">
+        <v>139</v>
+      </c>
+      <c r="D34" s="5">
+        <v>46227.0</v>
+      </c>
+      <c r="E34" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="F34" s="7" t="s">
+        <v>118</v>
+      </c>
+      <c r="G34" s="12" t="s">
+        <v>58</v>
+      </c>
+      <c r="H34" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="I34" s="6" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="35" ht="22.5" customHeight="1">
+      <c r="A35" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="F5" s="5" t="s">
-        <v>32</v>
-      </c>
-      <c r="G5" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="H5" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="I5" s="4" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="6" ht="22.5" customHeight="1">
-      <c r="A6" s="2" t="s">
+      <c r="B35" s="4" t="s">
+        <v>140</v>
+      </c>
+      <c r="C35" s="4" t="s">
+        <v>140</v>
+      </c>
+      <c r="D35" s="5">
+        <v>46227.0</v>
+      </c>
+      <c r="E35" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="F35" s="7" t="s">
+        <v>118</v>
+      </c>
+      <c r="G35" s="12" t="s">
+        <v>58</v>
+      </c>
+      <c r="H35" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="J35" s="6" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="36" ht="22.5" customHeight="1">
+      <c r="A36" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="B6" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="D6" s="3">
-        <v>46226.0</v>
-      </c>
-      <c r="E6" s="4" t="s">
+      <c r="B36" s="4" t="s">
+        <v>141</v>
+      </c>
+      <c r="C36" s="4" t="s">
+        <v>142</v>
+      </c>
+      <c r="D36" s="5">
+        <v>46227.0</v>
+      </c>
+      <c r="E36" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="F36" s="7" t="s">
+        <v>118</v>
+      </c>
+      <c r="G36" s="12" t="s">
+        <v>58</v>
+      </c>
+      <c r="H36" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="I36" s="6" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="37" ht="22.5" customHeight="1">
+      <c r="A37" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="F6" s="5" t="s">
-        <v>43</v>
-      </c>
-      <c r="G6" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="H6" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="I6" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="J6" s="4" t="s">
+      <c r="B37" s="4" t="s">
+        <v>143</v>
+      </c>
+      <c r="C37" s="4" t="s">
+        <v>143</v>
+      </c>
+      <c r="D37" s="5">
+        <v>46227.0</v>
+      </c>
+      <c r="E37" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="F37" s="7" t="s">
+        <v>118</v>
+      </c>
+      <c r="G37" s="12" t="s">
+        <v>58</v>
+      </c>
+      <c r="H37" s="6" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="7" ht="22.5" customHeight="1">
-      <c r="A7" s="2" t="s">
+      <c r="J37" s="6" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="38" ht="22.5" customHeight="1">
+      <c r="A38" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="B7" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="D7" s="3">
-        <v>46226.0</v>
-      </c>
-      <c r="E7" s="4" t="s">
+      <c r="B38" s="4" t="s">
+        <v>144</v>
+      </c>
+      <c r="C38" s="4" t="s">
+        <v>145</v>
+      </c>
+      <c r="D38" s="5">
+        <v>46227.0</v>
+      </c>
+      <c r="E38" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="F38" s="7" t="s">
+        <v>118</v>
+      </c>
+      <c r="G38" s="12" t="s">
+        <v>58</v>
+      </c>
+      <c r="H38" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="I38" s="6" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="39" ht="22.5" customHeight="1">
+      <c r="A39" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="F7" s="5" t="s">
-        <v>43</v>
-      </c>
-      <c r="G7" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="H7" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="I7" s="4" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="8" ht="22.5" customHeight="1">
-      <c r="A8" s="2" t="s">
+      <c r="B39" s="4" t="s">
+        <v>146</v>
+      </c>
+      <c r="C39" s="4" t="s">
+        <v>146</v>
+      </c>
+      <c r="D39" s="5">
+        <v>46227.0</v>
+      </c>
+      <c r="E39" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="F39" s="7" t="s">
+        <v>118</v>
+      </c>
+      <c r="G39" s="12" t="s">
+        <v>58</v>
+      </c>
+      <c r="H39" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="J39" s="6" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="40" ht="22.5" customHeight="1">
+      <c r="A40" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="B8" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="C8" s="2" t="s">
-        <v>50</v>
-      </c>
-      <c r="D8" s="3">
-        <v>46226.0</v>
-      </c>
-      <c r="E8" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="F8" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="G8" s="4" t="s">
+      <c r="B40" s="4" t="s">
+        <v>147</v>
+      </c>
+      <c r="C40" s="4" t="s">
+        <v>148</v>
+      </c>
+      <c r="D40" s="5">
+        <v>46227.0</v>
+      </c>
+      <c r="E40" s="6" t="s">
         <v>55</v>
       </c>
-      <c r="H8" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="I8" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="J8" s="4" t="s">
+      <c r="F40" s="7" t="s">
+        <v>118</v>
+      </c>
+      <c r="G40" s="12" t="s">
+        <v>58</v>
+      </c>
+      <c r="H40" s="6" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="9" ht="22.5" customHeight="1">
-      <c r="A9" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="B9" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="C9" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="D9" s="3">
-        <v>46226.0</v>
-      </c>
-      <c r="E9" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="F9" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="G9" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="H9" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="I9" s="4" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="10" ht="22.5" customHeight="1">
-      <c r="A10" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="B10" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="C10" s="2" t="s">
-        <v>62</v>
-      </c>
-      <c r="D10" s="3">
-        <v>46162.0</v>
-      </c>
-      <c r="E10" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="F10" s="5" t="s">
-        <v>63</v>
-      </c>
-      <c r="G10" s="4" t="s">
-        <v>66</v>
-      </c>
-      <c r="H10" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="I10" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="J10" s="4" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="11" ht="22.5" customHeight="1">
-      <c r="A11" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="B11" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="C11" s="2" t="s">
-        <v>69</v>
-      </c>
-      <c r="D11" s="3">
-        <v>46162.0</v>
-      </c>
-      <c r="E11" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="F11" s="5" t="s">
-        <v>63</v>
-      </c>
-      <c r="G11" s="4" t="s">
-        <v>66</v>
-      </c>
-      <c r="H11" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="I11" s="4" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="12" ht="22.5" customHeight="1">
-      <c r="A12" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="B12" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="C12" s="2" t="s">
-        <v>72</v>
-      </c>
-      <c r="D12" s="3">
-        <v>46162.0</v>
-      </c>
-      <c r="E12" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="F12" s="5" t="s">
-        <v>73</v>
-      </c>
-      <c r="G12" s="4" t="s">
-        <v>74</v>
-      </c>
-      <c r="H12" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="I12" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="J12" s="4" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="13" ht="22.5" customHeight="1">
-      <c r="A13" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="B13" s="2" t="s">
-        <v>75</v>
-      </c>
-      <c r="C13" s="4" t="s">
-        <v>76</v>
-      </c>
-      <c r="D13" s="3">
-        <v>46162.0</v>
-      </c>
-      <c r="E13" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="F13" s="5" t="s">
-        <v>73</v>
-      </c>
-      <c r="G13" s="4" t="s">
-        <v>74</v>
-      </c>
-      <c r="H13" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="I13" s="4" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="14" ht="22.5" customHeight="1">
-      <c r="A14" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="B14" s="2" t="s">
-        <v>77</v>
-      </c>
-      <c r="C14" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="D14" s="3">
-        <v>46162.0</v>
-      </c>
-      <c r="E14" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="F14" s="5" t="s">
-        <v>79</v>
-      </c>
-      <c r="G14" s="4" t="s">
-        <v>80</v>
-      </c>
-      <c r="H14" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="I14" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="J14" s="4" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="15" ht="22.5" customHeight="1">
-      <c r="A15" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="B15" s="2" t="s">
-        <v>81</v>
-      </c>
-      <c r="C15" s="4" t="s">
-        <v>82</v>
-      </c>
-      <c r="D15" s="3">
-        <v>46162.0</v>
-      </c>
-      <c r="E15" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="F15" s="5" t="s">
-        <v>79</v>
-      </c>
-      <c r="G15" s="4" t="s">
-        <v>80</v>
-      </c>
-      <c r="H15" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="I15" s="4" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="16" ht="22.5" customHeight="1">
-      <c r="A16" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="B16" s="2" t="s">
-        <v>83</v>
-      </c>
-      <c r="C16" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="D16" s="3">
-        <v>46162.0</v>
-      </c>
-      <c r="E16" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="F16" s="5" t="s">
-        <v>85</v>
-      </c>
-      <c r="G16" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="H16" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="I16" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="J16" s="4" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="17" ht="22.5" customHeight="1">
-      <c r="A17" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="B17" s="2" t="s">
-        <v>86</v>
-      </c>
-      <c r="C17" s="2" t="s">
-        <v>87</v>
-      </c>
-      <c r="D17" s="3">
-        <v>46162.0</v>
-      </c>
-      <c r="E17" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="F17" s="5" t="s">
-        <v>85</v>
-      </c>
-      <c r="G17" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="H17" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="I17" s="4" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="18" ht="22.5" customHeight="1">
-      <c r="A18" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="B18" s="2" t="s">
-        <v>88</v>
-      </c>
-      <c r="C18" s="2" t="s">
-        <v>89</v>
-      </c>
-      <c r="D18" s="3">
-        <v>46162.0</v>
-      </c>
-      <c r="E18" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="F18" s="5" t="s">
-        <v>90</v>
-      </c>
-      <c r="G18" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="H18" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="I18" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="J18" s="4" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="19" ht="22.5" customHeight="1">
-      <c r="A19" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="B19" s="2" t="s">
-        <v>91</v>
-      </c>
-      <c r="C19" s="4" t="s">
-        <v>92</v>
-      </c>
-      <c r="D19" s="3">
-        <v>46162.0</v>
-      </c>
-      <c r="E19" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="F19" s="5" t="s">
-        <v>90</v>
-      </c>
-      <c r="G19" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="H19" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="I19" s="4" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="20" ht="22.5" customHeight="1">
-      <c r="A20" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="B20" s="12" t="s">
-        <v>93</v>
-      </c>
-      <c r="C20" s="12" t="s">
-        <v>93</v>
-      </c>
-      <c r="D20" s="3">
-        <v>46227.0</v>
-      </c>
-      <c r="E20" s="4" t="s">
-        <v>56</v>
-      </c>
-      <c r="F20" s="13" t="s">
-        <v>94</v>
-      </c>
-      <c r="G20" s="14" t="s">
-        <v>95</v>
-      </c>
-      <c r="H20" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="J20" s="4" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="21" ht="22.5" customHeight="1">
-      <c r="A21" s="15" t="s">
-        <v>53</v>
-      </c>
-      <c r="B21" s="7" t="s">
-        <v>96</v>
-      </c>
-      <c r="C21" s="12" t="s">
-        <v>93</v>
-      </c>
-      <c r="D21" s="16">
-        <v>46227.0</v>
-      </c>
-      <c r="E21" s="17" t="s">
-        <v>56</v>
-      </c>
-      <c r="F21" s="18" t="s">
-        <v>97</v>
-      </c>
-      <c r="G21" s="19" t="s">
-        <v>95</v>
-      </c>
-      <c r="H21" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="I21" s="20" t="s">
-        <v>98</v>
-      </c>
-      <c r="J21" s="21" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="22" ht="22.5" customHeight="1">
-      <c r="A22" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="B22" s="22" t="s">
-        <v>99</v>
-      </c>
-      <c r="C22" s="22" t="s">
-        <v>100</v>
-      </c>
-      <c r="D22" s="3">
-        <v>46227.0</v>
-      </c>
-      <c r="E22" s="4" t="s">
-        <v>56</v>
-      </c>
-      <c r="F22" s="5" t="s">
-        <v>94</v>
-      </c>
-      <c r="G22" s="14" t="s">
-        <v>95</v>
-      </c>
-      <c r="H22" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="I22" s="4" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="23" ht="22.5" customHeight="1">
-      <c r="A23" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="B23" s="12" t="s">
-        <v>102</v>
-      </c>
-      <c r="C23" s="12" t="s">
-        <v>102</v>
-      </c>
-      <c r="D23" s="3">
-        <v>46227.0</v>
-      </c>
-      <c r="E23" s="4" t="s">
-        <v>56</v>
-      </c>
-      <c r="F23" s="5" t="s">
-        <v>94</v>
-      </c>
-      <c r="G23" s="14" t="s">
-        <v>95</v>
-      </c>
-      <c r="H23" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="J23" s="4" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="24" ht="22.5" customHeight="1">
-      <c r="A24" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="B24" s="22" t="s">
-        <v>103</v>
-      </c>
-      <c r="C24" s="22" t="s">
-        <v>104</v>
-      </c>
-      <c r="D24" s="3">
-        <v>46227.0</v>
-      </c>
-      <c r="E24" s="4" t="s">
-        <v>56</v>
-      </c>
-      <c r="F24" s="5" t="s">
-        <v>94</v>
-      </c>
-      <c r="G24" s="14" t="s">
-        <v>95</v>
-      </c>
-      <c r="H24" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="I24" s="4" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="25" ht="22.5" customHeight="1">
-      <c r="A25" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="B25" s="12" t="s">
-        <v>105</v>
-      </c>
-      <c r="C25" s="23" t="s">
-        <v>105</v>
-      </c>
-      <c r="D25" s="3">
-        <v>46227.0</v>
-      </c>
-      <c r="E25" s="4" t="s">
-        <v>56</v>
-      </c>
-      <c r="F25" s="5" t="s">
-        <v>94</v>
-      </c>
-      <c r="G25" s="14" t="s">
-        <v>95</v>
-      </c>
-      <c r="H25" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="J25" s="4" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="26" ht="22.5" customHeight="1">
-      <c r="A26" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="B26" s="24" t="s">
-        <v>106</v>
-      </c>
-      <c r="C26" s="24" t="s">
-        <v>107</v>
-      </c>
-      <c r="D26" s="3">
-        <v>46227.0</v>
-      </c>
-      <c r="E26" s="4" t="s">
-        <v>56</v>
-      </c>
-      <c r="F26" s="5" t="s">
-        <v>94</v>
-      </c>
-      <c r="G26" s="14" t="s">
-        <v>95</v>
-      </c>
-      <c r="H26" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="I26" s="4" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="27" ht="22.5" customHeight="1">
-      <c r="A27" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="B27" s="12" t="s">
-        <v>108</v>
-      </c>
-      <c r="C27" s="12" t="s">
-        <v>108</v>
-      </c>
-      <c r="D27" s="3">
-        <v>46227.0</v>
-      </c>
-      <c r="E27" s="4" t="s">
-        <v>56</v>
-      </c>
-      <c r="F27" s="5" t="s">
-        <v>94</v>
-      </c>
-      <c r="G27" s="14" t="s">
-        <v>95</v>
-      </c>
-      <c r="H27" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="J27" s="4" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="28" ht="22.5" customHeight="1">
-      <c r="A28" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="B28" s="12" t="s">
-        <v>109</v>
-      </c>
-      <c r="C28" s="12" t="s">
-        <v>110</v>
-      </c>
-      <c r="D28" s="3">
-        <v>46227.0</v>
-      </c>
-      <c r="E28" s="4" t="s">
-        <v>56</v>
-      </c>
-      <c r="F28" s="5" t="s">
-        <v>94</v>
-      </c>
-      <c r="G28" s="14" t="s">
-        <v>95</v>
-      </c>
-      <c r="H28" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="I28" s="4" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="29" ht="22.5" customHeight="1">
-      <c r="A29" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="B29" s="2" t="s">
-        <v>111</v>
-      </c>
-      <c r="C29" s="2" t="s">
-        <v>111</v>
-      </c>
-      <c r="D29" s="3">
-        <v>46227.0</v>
-      </c>
-      <c r="E29" s="4" t="s">
-        <v>56</v>
-      </c>
-      <c r="F29" s="5" t="s">
-        <v>97</v>
-      </c>
-      <c r="G29" s="14" t="s">
-        <v>95</v>
-      </c>
-      <c r="H29" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="J29" s="4" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="30" ht="22.5" customHeight="1">
-      <c r="A30" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="B30" s="7" t="s">
-        <v>112</v>
-      </c>
-      <c r="C30" s="2" t="s">
-        <v>111</v>
-      </c>
-      <c r="D30" s="3">
-        <v>46227.0</v>
-      </c>
-      <c r="E30" s="4" t="s">
-        <v>56</v>
-      </c>
-      <c r="F30" s="5" t="s">
-        <v>97</v>
-      </c>
-      <c r="G30" s="14" t="s">
-        <v>95</v>
-      </c>
-      <c r="H30" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="I30" s="25" t="s">
-        <v>98</v>
-      </c>
-      <c r="J30" s="4" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="31" ht="22.5" customHeight="1">
-      <c r="A31" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="B31" s="2" t="s">
-        <v>113</v>
-      </c>
-      <c r="C31" s="26" t="s">
-        <v>114</v>
-      </c>
-      <c r="D31" s="3">
-        <v>46227.0</v>
-      </c>
-      <c r="E31" s="4" t="s">
-        <v>56</v>
-      </c>
-      <c r="F31" s="5" t="s">
-        <v>97</v>
-      </c>
-      <c r="G31" s="14" t="s">
-        <v>95</v>
-      </c>
-      <c r="H31" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="I31" s="4" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="32" ht="22.5" customHeight="1">
-      <c r="A32" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="B32" s="2" t="s">
-        <v>115</v>
-      </c>
-      <c r="C32" s="2" t="s">
-        <v>115</v>
-      </c>
-      <c r="D32" s="3">
-        <v>46227.0</v>
-      </c>
-      <c r="E32" s="4" t="s">
-        <v>56</v>
-      </c>
-      <c r="F32" s="5" t="s">
-        <v>97</v>
-      </c>
-      <c r="G32" s="14" t="s">
-        <v>95</v>
-      </c>
-      <c r="H32" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="J32" s="4" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="33" ht="22.5" customHeight="1">
-      <c r="A33" s="27" t="s">
-        <v>53</v>
-      </c>
-      <c r="B33" s="7" t="s">
-        <v>116</v>
-      </c>
-      <c r="C33" s="2" t="s">
-        <v>115</v>
-      </c>
-      <c r="D33" s="28">
-        <v>46227.0</v>
-      </c>
-      <c r="E33" s="29" t="s">
-        <v>56</v>
-      </c>
-      <c r="F33" s="30" t="s">
-        <v>97</v>
-      </c>
-      <c r="G33" s="31" t="s">
-        <v>95</v>
-      </c>
-      <c r="H33" s="29" t="s">
-        <v>26</v>
-      </c>
-      <c r="I33" s="32" t="s">
-        <v>98</v>
-      </c>
-      <c r="J33" s="33" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="34" ht="22.5" customHeight="1">
-      <c r="A34" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="B34" s="2" t="s">
-        <v>117</v>
-      </c>
-      <c r="C34" s="4" t="s">
-        <v>118</v>
-      </c>
-      <c r="D34" s="3">
-        <v>46227.0</v>
-      </c>
-      <c r="E34" s="4" t="s">
-        <v>56</v>
-      </c>
-      <c r="F34" s="5" t="s">
-        <v>97</v>
-      </c>
-      <c r="G34" s="14" t="s">
-        <v>95</v>
-      </c>
-      <c r="H34" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="I34" s="4" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="35" ht="22.5" customHeight="1">
-      <c r="A35" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="B35" s="2" t="s">
-        <v>119</v>
-      </c>
-      <c r="C35" s="2" t="s">
-        <v>119</v>
-      </c>
-      <c r="D35" s="3">
-        <v>46227.0</v>
-      </c>
-      <c r="E35" s="4" t="s">
-        <v>56</v>
-      </c>
-      <c r="F35" s="5" t="s">
-        <v>97</v>
-      </c>
-      <c r="G35" s="14" t="s">
-        <v>95</v>
-      </c>
-      <c r="H35" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="J35" s="4" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="36" ht="22.5" customHeight="1">
-      <c r="A36" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="B36" s="2" t="s">
-        <v>120</v>
-      </c>
-      <c r="C36" s="2" t="s">
-        <v>121</v>
-      </c>
-      <c r="D36" s="3">
-        <v>46227.0</v>
-      </c>
-      <c r="E36" s="4" t="s">
-        <v>56</v>
-      </c>
-      <c r="F36" s="5" t="s">
-        <v>97</v>
-      </c>
-      <c r="G36" s="14" t="s">
-        <v>95</v>
-      </c>
-      <c r="H36" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="I36" s="4" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="37" ht="22.5" customHeight="1">
-      <c r="A37" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="B37" s="2" t="s">
+      <c r="I40" s="6" t="s">
         <v>122</v>
-      </c>
-      <c r="C37" s="2" t="s">
-        <v>122</v>
-      </c>
-      <c r="D37" s="3">
-        <v>46227.0</v>
-      </c>
-      <c r="E37" s="4" t="s">
-        <v>56</v>
-      </c>
-      <c r="F37" s="5" t="s">
-        <v>97</v>
-      </c>
-      <c r="G37" s="14" t="s">
-        <v>95</v>
-      </c>
-      <c r="H37" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="J37" s="4" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="38" ht="22.5" customHeight="1">
-      <c r="A38" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="B38" s="2" t="s">
-        <v>123</v>
-      </c>
-      <c r="C38" s="2" t="s">
-        <v>124</v>
-      </c>
-      <c r="D38" s="3">
-        <v>46227.0</v>
-      </c>
-      <c r="E38" s="4" t="s">
-        <v>56</v>
-      </c>
-      <c r="F38" s="5" t="s">
-        <v>97</v>
-      </c>
-      <c r="G38" s="14" t="s">
-        <v>95</v>
-      </c>
-      <c r="H38" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="I38" s="4" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="39" ht="22.5" customHeight="1">
-      <c r="A39" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="B39" s="2" t="s">
-        <v>125</v>
-      </c>
-      <c r="C39" s="2" t="s">
-        <v>125</v>
-      </c>
-      <c r="D39" s="3">
-        <v>46227.0</v>
-      </c>
-      <c r="E39" s="4" t="s">
-        <v>56</v>
-      </c>
-      <c r="F39" s="5" t="s">
-        <v>97</v>
-      </c>
-      <c r="G39" s="14" t="s">
-        <v>95</v>
-      </c>
-      <c r="H39" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="J39" s="4" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="40" ht="22.5" customHeight="1">
-      <c r="A40" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="B40" s="2" t="s">
-        <v>126</v>
-      </c>
-      <c r="C40" s="2" t="s">
-        <v>127</v>
-      </c>
-      <c r="D40" s="3">
-        <v>46227.0</v>
-      </c>
-      <c r="E40" s="4" t="s">
-        <v>56</v>
-      </c>
-      <c r="F40" s="5" t="s">
-        <v>97</v>
-      </c>
-      <c r="G40" s="14" t="s">
-        <v>95</v>
-      </c>
-      <c r="H40" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="I40" s="4" t="s">
-        <v>101</v>
       </c>
     </row>
     <row r="41" ht="15.75" customHeight="1"/>

</xml_diff>

<commit_message>
Fix typo in data README and files provenance file
</commit_message>
<xml_diff>
--- a/data/files_provenance_ECCB-2026-T6.xlsx
+++ b/data/files_provenance_ECCB-2026-T6.xlsx
@@ -10,7 +10,7 @@
   <calcPr/>
   <extLst>
     <ext uri="GoogleSheetsCustomDataVersion2">
-      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId6" roundtripDataChecksum="GKSCo0ojxI8ZjUlxdoIabpxHFONFuc30jw5nNNAgWGk="/>
+      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId6" roundtripDataChecksum="Ugc4rKcaPgtpvzq7RTdx3umEwMpD/wFu9qPvXQvgekY="/>
     </ext>
   </extLst>
 </workbook>
@@ -37,15 +37,15 @@
     <t>Source</t>
   </si>
   <si>
+    <t>Release</t>
+  </si>
+  <si>
+    <t>Assembly</t>
+  </si>
+  <si>
     <t>Version</t>
   </si>
   <si>
-    <t>Release</t>
-  </si>
-  <si>
-    <t>Assembly</t>
-  </si>
-  <si>
     <t>Filters/processing</t>
   </si>
   <si>
@@ -55,24 +55,24 @@
     <t>Ensembl_Regulation</t>
   </si>
   <si>
+    <t>GRCh38-cCRE-colors18062026.bed.gz</t>
+  </si>
+  <si>
+    <t>GRCh38-cCREs.bed</t>
+  </si>
+  <si>
     <t>ENCODE</t>
   </si>
   <si>
-    <t>GRCh38-cCRE-colors18062026.bed.gz</t>
-  </si>
-  <si>
-    <t>GRCh38-cCREs.bed</t>
-  </si>
-  <si>
     <t>ENCFF345CWR.atac.bed</t>
   </si>
   <si>
+    <t>ENCODE SCREEN</t>
+  </si>
+  <si>
     <t>ENCFF345CWR.bed</t>
   </si>
   <si>
-    <t>ENCODE SCREEN</t>
-  </si>
-  <si>
     <t>https://screen.wenglab.org/downloads</t>
   </si>
   <si>
@@ -82,42 +82,42 @@
     <t>V4</t>
   </si>
   <si>
+    <t>GRCh38</t>
+  </si>
+  <si>
+    <t>Added feature colors. Gzip compression</t>
+  </si>
+  <si>
     <t>ENCODE4 v1.8.0</t>
   </si>
   <si>
-    <t>GRCh38</t>
-  </si>
-  <si>
-    <t>Added feature colors. Gzip compression</t>
+    <t>0-based</t>
   </si>
   <si>
     <t>mm10</t>
   </si>
   <si>
-    <t>0-based</t>
-  </si>
-  <si>
     <t>Rename to include assay type</t>
   </si>
   <si>
+    <t>GRCh38-cCRE-colors18062026.bed.idx</t>
+  </si>
+  <si>
     <t>ENCFF633ETU.atac.chr6.5911252-7710120.bw</t>
   </si>
   <si>
+    <t>GRCh38-cCRE-colors18062026.bed</t>
+  </si>
+  <si>
     <t>ENCFF633ETU.bigWig</t>
   </si>
   <si>
-    <t>GRCh38-cCRE-colors18062026.bed.idx</t>
-  </si>
-  <si>
-    <t>GRCh38-cCRE-colors18062026.bed</t>
+    <t>Bed file index</t>
   </si>
   <si>
     <t xml:space="preserve">Rename to include assay type. Trimming </t>
   </si>
   <si>
-    <t>Bed file index</t>
-  </si>
-  <si>
     <t>ENCFF053ITU.k27ac.bed</t>
   </si>
   <si>
@@ -136,6 +136,12 @@
     <t>GRCm39</t>
   </si>
   <si>
+    <t>Liftover from mm10, add feature colors. Gzip compression</t>
+  </si>
+  <si>
+    <t>mm10-cCRE-colors18062026.bed.gz</t>
+  </si>
+  <si>
     <t>ENCODE4 v1.5.1</t>
   </si>
   <si>
@@ -145,10 +151,10 @@
     <t>ENCFF607CHT.bigWig</t>
   </si>
   <si>
-    <t>Liftover from mm10, add feature colors. Gzip compression</t>
-  </si>
-  <si>
-    <t>mm10-cCRE-colors18062026.bed.gz</t>
+    <t>HCT116-cCRE.chr8.bed</t>
+  </si>
+  <si>
+    <t>ENCFF431JDU_ENCFF964OOU_ENCFF787LMI_ENCFF388PVO.bed</t>
   </si>
   <si>
     <t>ENCFF079TUC.k4me3.bed</t>
@@ -160,10 +166,10 @@
     <t>https://www.encodeproject.org/experiments/ENCSR835BZO/</t>
   </si>
   <si>
-    <t>HCT116-cCRE.chr8.bed</t>
-  </si>
-  <si>
-    <t>ENCFF431JDU_ENCFF964OOU_ENCFF787LMI_ENCFF388PVO.bed</t>
+    <t>Filter chr8 features. Rename. Gzip compression.</t>
+  </si>
+  <si>
+    <t>Homo_sapiens.GRCh38.regulatory_features.v116.bb</t>
   </si>
   <si>
     <t>ENCFF798ETE.k4me3.chr6.5911252-7710120.bw</t>
@@ -172,57 +178,51 @@
     <t>ENCFF798ETE.bigWig</t>
   </si>
   <si>
-    <t>Filter chr8 features. Rename. Gzip compression.</t>
+    <t>Ensembl Regulation</t>
+  </si>
+  <si>
+    <t>https://regulation.ensembl.org/regulatory_features/homo_sapiens</t>
   </si>
   <si>
     <t>ENCFF217ZPW.k4me1.bed</t>
   </si>
   <si>
-    <t>Homo_sapiens.GRCh38.regulatory_features.v116.bb</t>
-  </si>
-  <si>
     <t>ENCFF217ZPW.bed</t>
   </si>
   <si>
-    <t>Ensembl Regulation</t>
-  </si>
-  <si>
-    <t>https://regulation.ensembl.org/regulatory_features/homo_sapiens</t>
+    <t>2025-12</t>
   </si>
   <si>
     <t>https://www.encodeproject.org/experiments/ENCSR496TBX/</t>
   </si>
   <si>
-    <t>2025-12</t>
+    <t>Homo_sapiens.GRCh38.regulatory_features.v116.gff3.gz</t>
   </si>
   <si>
     <t>ENCODE4 v1.6.1</t>
   </si>
   <si>
-    <t>Homo_sapiens.GRCh38.regulatory_features.v116.gff3.gz</t>
-  </si>
-  <si>
     <t>ENCFF013ALT.k4me1.chr6.5911252-7710120.bw</t>
   </si>
   <si>
+    <t>1-based</t>
+  </si>
+  <si>
     <t>ENCFF013ALT.bigWig</t>
   </si>
   <si>
-    <t>1-based</t>
-  </si>
-  <si>
     <t>Mus_musculus.GRCm39.regulatory_features.v116.bb</t>
   </si>
   <si>
+    <t>https://regulation.ensembl.org/regulatory_features/mus_musculus</t>
+  </si>
+  <si>
     <t>ENCFF240LRP.dnase.bed</t>
   </si>
   <si>
     <t>ENCFF240LRP.bed</t>
   </si>
   <si>
-    <t>https://regulation.ensembl.org/regulatory_features/mus_musculus</t>
-  </si>
-  <si>
     <t>https://www.encodeproject.org/experiments/ENCSR000ENM/</t>
   </si>
   <si>
@@ -241,42 +241,42 @@
     <t>Vista</t>
   </si>
   <si>
+    <t>vistaEnhancers_GRCh38.bb</t>
+  </si>
+  <si>
+    <t>vistaEnhancers.bb</t>
+  </si>
+  <si>
     <t>ENCFF296ZZB.atac.bed</t>
   </si>
   <si>
-    <t>vistaEnhancers_GRCh38.bb</t>
+    <t>UCSC</t>
   </si>
   <si>
     <t>ENCFF296ZZB.bed</t>
   </si>
   <si>
-    <t>vistaEnhancers.bb</t>
+    <t>https://hgdownload.soe.ucsc.edu/gbdb/hg38/vistaEnhancers/</t>
   </si>
   <si>
     <t>https://www.encodeproject.org/experiments/ENCSR872WGW/</t>
   </si>
   <si>
-    <t>UCSC</t>
-  </si>
-  <si>
-    <t>https://hgdownload.soe.ucsc.edu/gbdb/hg38/vistaEnhancers/</t>
-  </si>
-  <si>
     <t>ENCODE4 v1.9.1</t>
   </si>
   <si>
     <t>01/07/2026</t>
   </si>
   <si>
+    <t>Rename</t>
+  </si>
+  <si>
     <t>ENCFF624HRW.atac.chr8.126229903-128914986.bw</t>
   </si>
   <si>
     <t>ENCFF624HRW.bw</t>
   </si>
   <si>
-    <t>Rename</t>
-  </si>
-  <si>
     <t>Fantom5</t>
   </si>
   <si>
@@ -298,34 +298,34 @@
     <t>ENCFF711MPL.bed</t>
   </si>
   <si>
+    <t>V9</t>
+  </si>
+  <si>
     <t>https://www.encodeproject.org/experiments/ENCSR333OPW/</t>
   </si>
   <si>
-    <t>V9</t>
-  </si>
-  <si>
     <t>Gzip compression.</t>
   </si>
   <si>
+    <t>RefSeq</t>
+  </si>
+  <si>
     <t xml:space="preserve">ENCODE4 v1.5.1 </t>
   </si>
   <si>
-    <t>RefSeq</t>
-  </si>
-  <si>
     <t>GCF_000001405.40_GRCh38.p14_genomic.RefSeqFE.gff.gz</t>
   </si>
   <si>
     <t>GCF_000001405.40_GRCh38.p14_genomic.gff</t>
   </si>
   <si>
+    <t>https://ftp.ncbi.nlm.nih.gov/genomes/refseq/vertebrate_mammalian/Homo_sapiens/latest_assembly_versions/GCF_000001405.40_GRCh38.p14/</t>
+  </si>
+  <si>
     <t>ENCFF394IMO.k4me3.chr8.126229903-128914986.bw</t>
   </si>
   <si>
     <t>ENCFF394IMO.bw</t>
-  </si>
-  <si>
-    <t>https://ftp.ncbi.nlm.nih.gov/genomes/refseq/vertebrate_mammalian/Homo_sapiens/latest_assembly_versions/GCF_000001405.40_GRCh38.p14/</t>
   </si>
   <si>
     <t>08/01/2025</t>
@@ -817,13 +817,13 @@
     </dxf>
   </dxfs>
   <tableStyles count="2">
-    <tableStyle count="4" pivot="0" name="CREs annotation-style">
+    <tableStyle count="4" pivot="0" name="Evidence-style">
       <tableStyleElement dxfId="1" type="headerRow"/>
       <tableStyleElement dxfId="2" type="firstRowStripe"/>
       <tableStyleElement dxfId="3" type="secondRowStripe"/>
       <tableStyleElement dxfId="4" size="0" type="wholeTable"/>
     </tableStyle>
-    <tableStyle count="4" pivot="0" name="Evidence-style">
+    <tableStyle count="4" pivot="0" name="CREs annotation-style">
       <tableStyleElement dxfId="1" type="headerRow"/>
       <tableStyleElement dxfId="2" type="firstRowStripe"/>
       <tableStyleElement dxfId="3" type="secondRowStripe"/>
@@ -842,7 +842,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:J13" displayName="Table2" name="Table2" id="2">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:J13" displayName="Table2" name="Table2" id="1">
   <tableColumns count="10">
     <tableColumn name="Folder" id="1"/>
     <tableColumn name="File name" id="2"/>
@@ -860,7 +860,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:J40" displayName="Table1" name="Table1" id="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:J40" displayName="Table1" name="Table1" id="2">
   <tableColumns count="10">
     <tableColumn name="Folder" id="1"/>
     <tableColumn name="File name" id="2"/>
@@ -1110,10 +1110,10 @@
         <v>5</v>
       </c>
       <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="1" t="s">
         <v>7</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>8</v>
       </c>
       <c r="I1" s="1" t="s">
         <v>9</v>
@@ -1127,16 +1127,16 @@
         <v>11</v>
       </c>
       <c r="B2" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C2" s="4" t="s">
         <v>13</v>
-      </c>
-      <c r="C2" s="4" t="s">
-        <v>14</v>
       </c>
       <c r="D2" s="5">
         <v>46191.0</v>
       </c>
       <c r="E2" s="6" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F2" s="7" t="s">
         <v>18</v>
@@ -1145,44 +1145,44 @@
         <v>20</v>
       </c>
       <c r="H2" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="I2" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="I2" s="9" t="s">
-        <v>23</v>
-      </c>
       <c r="J2" s="6" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="3" ht="22.5" customHeight="1">
       <c r="A3" s="2" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B3" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="C3" s="4" t="s">
         <v>29</v>
-      </c>
-      <c r="C3" s="4" t="s">
-        <v>30</v>
       </c>
       <c r="D3" s="5"/>
       <c r="E3" s="6" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F3" s="10"/>
       <c r="G3" s="8" t="s">
         <v>20</v>
       </c>
       <c r="H3" s="9" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="I3" s="9" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="J3" s="6"/>
     </row>
     <row r="4" ht="22.5" customHeight="1">
       <c r="A4" s="11" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B4" s="3" t="s">
         <v>35</v>
@@ -1194,7 +1194,7 @@
         <v>46191.0</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F4" s="7" t="s">
         <v>18</v>
@@ -1206,18 +1206,18 @@
         <v>38</v>
       </c>
       <c r="I4" s="9" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="J4" s="6" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="5" ht="22.5" customHeight="1">
       <c r="A5" s="11" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="C5" s="4" t="s">
         <v>36</v>
@@ -1226,7 +1226,7 @@
         <v>46191.0</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F5" s="7" t="s">
         <v>18</v>
@@ -1235,30 +1235,30 @@
         <v>20</v>
       </c>
       <c r="H5" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="I5" s="9" t="s">
+        <v>22</v>
+      </c>
+      <c r="J5" s="6" t="s">
         <v>24</v>
-      </c>
-      <c r="I5" s="9" t="s">
-        <v>23</v>
-      </c>
-      <c r="J5" s="6" t="s">
-        <v>25</v>
       </c>
     </row>
     <row r="6" ht="22.5" customHeight="1">
       <c r="A6" s="11" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="D6" s="5">
         <v>46227.0</v>
       </c>
       <c r="E6" s="6" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F6" s="7" t="s">
         <v>18</v>
@@ -1267,13 +1267,13 @@
         <v>20</v>
       </c>
       <c r="H6" s="6" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="I6" s="9" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="J6" s="6" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="7" ht="22.5" customHeight="1">
@@ -1281,28 +1281,28 @@
         <v>11</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="D7" s="5">
         <v>46206.0</v>
       </c>
       <c r="E7" s="6" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="F7" s="7" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="G7" s="12" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="H7" s="6" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="J7" s="6" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="8" ht="22.5" customHeight="1">
@@ -1310,28 +1310,28 @@
         <v>11</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D8" s="5">
         <v>46191.0</v>
       </c>
       <c r="E8" s="6" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="F8" s="7" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="G8" s="12" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="H8" s="6" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="J8" s="6" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="9" ht="22.5" customHeight="1">
@@ -1348,19 +1348,19 @@
         <v>46206.0</v>
       </c>
       <c r="E9" s="6" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="F9" s="13" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="G9" s="12" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="H9" s="6" t="s">
         <v>38</v>
       </c>
       <c r="J9" s="6" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="10" ht="22.5" customHeight="1">
@@ -1377,19 +1377,19 @@
         <v>46191.0</v>
       </c>
       <c r="E10" s="6" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="F10" s="13" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="G10" s="12" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="H10" s="6" t="s">
         <v>38</v>
       </c>
       <c r="J10" s="6" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="11" ht="15.75" customHeight="1">
@@ -1397,31 +1397,31 @@
         <v>73</v>
       </c>
       <c r="B11" s="15" t="s">
+        <v>74</v>
+      </c>
+      <c r="C11" s="16" t="s">
         <v>75</v>
-      </c>
-      <c r="C11" s="16" t="s">
-        <v>77</v>
       </c>
       <c r="D11" s="17">
         <v>46251.0</v>
       </c>
       <c r="E11" s="18" t="s">
+        <v>77</v>
+      </c>
+      <c r="F11" s="19" t="s">
         <v>79</v>
-      </c>
-      <c r="F11" s="19" t="s">
-        <v>80</v>
       </c>
       <c r="G11" s="20" t="s">
         <v>82</v>
       </c>
       <c r="H11" s="21" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="I11" s="22" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="J11" s="6" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="12" ht="15.75" customHeight="1">
@@ -1444,21 +1444,21 @@
         <v>90</v>
       </c>
       <c r="G12" s="24" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="H12" s="21" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="I12" s="23" t="s">
         <v>95</v>
       </c>
       <c r="J12" s="6" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="13" ht="15.75" customHeight="1">
       <c r="A13" s="14" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B13" s="23" t="s">
         <v>98</v>
@@ -1470,22 +1470,22 @@
         <v>46251.0</v>
       </c>
       <c r="E13" s="18" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="F13" s="19" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="G13" s="20" t="s">
         <v>103</v>
       </c>
       <c r="H13" s="21" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="I13" s="22" t="s">
         <v>104</v>
       </c>
       <c r="J13" s="21" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="14" ht="15.75" customHeight="1"/>
@@ -2478,11 +2478,11 @@
     <row r="1001" ht="15.75" customHeight="1"/>
   </sheetData>
   <dataValidations>
-    <dataValidation type="list" allowBlank="1" sqref="A2:A13">
-      <formula1>"ENCODE,Ensembl_Regulation,Vista,Fantom5,RefSeq"</formula1>
-    </dataValidation>
     <dataValidation type="custom" allowBlank="1" showDropDown="1" sqref="D2:D13">
       <formula1>OR(NOT(ISERROR(DATEVALUE(D2))), AND(ISNUMBER(D2), LEFT(CELL("format", D2))="D"))</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" sqref="A2:A13">
+      <formula1>"ENCODE,Ensembl_Regulation,VISTA,Fantom5,RefSeq"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showDropDown="1" showErrorMessage="1" sqref="J2:J13">
       <formula1>"0-based,1-based"</formula1>
@@ -2548,10 +2548,10 @@
         <v>5</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="I1" s="1" t="s">
         <v>9</v>
@@ -2562,68 +2562,68 @@
     </row>
     <row r="2" ht="22.5" customHeight="1">
       <c r="A2" s="4" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B2" s="4" t="s">
         <v>15</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D2" s="5">
         <v>46226.0</v>
       </c>
       <c r="E2" s="6" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="F2" s="7" t="s">
         <v>19</v>
       </c>
       <c r="G2" s="6" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="H2" s="6" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="I2" s="6" t="s">
         <v>26</v>
       </c>
       <c r="J2" s="6" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="3" ht="22.5" customHeight="1">
       <c r="A3" s="4" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="D3" s="5">
         <v>46226.0</v>
       </c>
       <c r="E3" s="6" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="F3" s="7" t="s">
         <v>19</v>
       </c>
       <c r="G3" s="6" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="H3" s="6" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="I3" s="6" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="4" ht="22.5" customHeight="1">
       <c r="A4" s="4" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B4" s="4" t="s">
         <v>33</v>
@@ -2635,190 +2635,190 @@
         <v>46226.0</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="F4" s="7" t="s">
         <v>37</v>
       </c>
       <c r="G4" s="6" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="H4" s="6" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="I4" s="6" t="s">
         <v>26</v>
       </c>
       <c r="J4" s="6" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="5" ht="22.5" customHeight="1">
       <c r="A5" s="4" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="D5" s="5">
         <v>46226.0</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="F5" s="7" t="s">
         <v>37</v>
       </c>
       <c r="G5" s="6" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="H5" s="6" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="I5" s="6" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="6" ht="22.5" customHeight="1">
       <c r="A6" s="4" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="D6" s="5">
         <v>46226.0</v>
       </c>
       <c r="E6" s="6" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="F6" s="7" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="G6" s="6" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="H6" s="6" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="I6" s="6" t="s">
         <v>26</v>
       </c>
       <c r="J6" s="6" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="7" ht="22.5" customHeight="1">
       <c r="A7" s="4" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="D7" s="5">
         <v>46226.0</v>
       </c>
       <c r="E7" s="6" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="F7" s="7" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="G7" s="6" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="H7" s="6" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="I7" s="6" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="8" ht="22.5" customHeight="1">
       <c r="A8" s="4" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="D8" s="5">
         <v>46226.0</v>
       </c>
       <c r="E8" s="6" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="F8" s="7" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="G8" s="6" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="H8" s="6" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="I8" s="6" t="s">
         <v>26</v>
       </c>
       <c r="J8" s="6" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="9" ht="22.5" customHeight="1">
       <c r="A9" s="4" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B9" s="4" t="s">
         <v>61</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D9" s="5">
         <v>46226.0</v>
       </c>
       <c r="E9" s="6" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="F9" s="7" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="G9" s="6" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="H9" s="6" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="I9" s="6" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="10" ht="22.5" customHeight="1">
       <c r="A10" s="4" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="D10" s="5">
         <v>46162.0</v>
       </c>
       <c r="E10" s="6" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="F10" s="7" t="s">
         <v>68</v>
@@ -2827,18 +2827,18 @@
         <v>69</v>
       </c>
       <c r="H10" s="6" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="I10" s="6" t="s">
         <v>26</v>
       </c>
       <c r="J10" s="6" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="11" ht="22.5" customHeight="1">
       <c r="A11" s="4" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B11" s="4" t="s">
         <v>71</v>
@@ -2850,7 +2850,7 @@
         <v>46162.0</v>
       </c>
       <c r="E11" s="6" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="F11" s="7" t="s">
         <v>68</v>
@@ -2859,76 +2859,76 @@
         <v>69</v>
       </c>
       <c r="H11" s="6" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="I11" s="6" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="12" ht="22.5" customHeight="1">
       <c r="A12" s="4" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="D12" s="5">
         <v>46162.0</v>
       </c>
       <c r="E12" s="6" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="F12" s="7" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="G12" s="6" t="s">
         <v>81</v>
       </c>
       <c r="H12" s="6" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="I12" s="6" t="s">
         <v>26</v>
       </c>
       <c r="J12" s="6" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="13" ht="22.5" customHeight="1">
       <c r="A13" s="4" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="D13" s="5">
         <v>46162.0</v>
       </c>
       <c r="E13" s="6" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="F13" s="7" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="G13" s="6" t="s">
         <v>81</v>
       </c>
       <c r="H13" s="6" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="I13" s="6" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="14" ht="22.5" customHeight="1">
       <c r="A14" s="4" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B14" s="4" t="s">
         <v>91</v>
@@ -2940,56 +2940,56 @@
         <v>46162.0</v>
       </c>
       <c r="E14" s="6" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="F14" s="7" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="G14" s="6" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="H14" s="6" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="I14" s="6" t="s">
         <v>26</v>
       </c>
       <c r="J14" s="6" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="15" ht="22.5" customHeight="1">
       <c r="A15" s="4" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="C15" s="6" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="D15" s="5">
         <v>46162.0</v>
       </c>
       <c r="E15" s="6" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="F15" s="7" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="G15" s="6" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="H15" s="6" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="I15" s="6" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="16" ht="22.5" customHeight="1">
       <c r="A16" s="4" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B16" s="4" t="s">
         <v>105</v>
@@ -3001,27 +3001,27 @@
         <v>46162.0</v>
       </c>
       <c r="E16" s="6" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="F16" s="7" t="s">
         <v>107</v>
       </c>
       <c r="G16" s="6" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="H16" s="6" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="I16" s="6" t="s">
         <v>26</v>
       </c>
       <c r="J16" s="6" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="17" ht="22.5" customHeight="1">
       <c r="A17" s="4" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B17" s="4" t="s">
         <v>108</v>
@@ -3033,24 +3033,24 @@
         <v>46162.0</v>
       </c>
       <c r="E17" s="6" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="F17" s="7" t="s">
         <v>107</v>
       </c>
       <c r="G17" s="6" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="H17" s="6" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="I17" s="6" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="18" ht="22.5" customHeight="1">
       <c r="A18" s="4" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B18" s="4" t="s">
         <v>110</v>
@@ -3062,27 +3062,27 @@
         <v>46162.0</v>
       </c>
       <c r="E18" s="6" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="F18" s="7" t="s">
         <v>112</v>
       </c>
       <c r="G18" s="6" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="H18" s="6" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="I18" s="6" t="s">
         <v>26</v>
       </c>
       <c r="J18" s="6" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="19" ht="22.5" customHeight="1">
       <c r="A19" s="4" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B19" s="4" t="s">
         <v>113</v>
@@ -3094,19 +3094,19 @@
         <v>46162.0</v>
       </c>
       <c r="E19" s="6" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="F19" s="7" t="s">
         <v>112</v>
       </c>
       <c r="G19" s="6" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="H19" s="6" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="I19" s="6" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="20" ht="22.5" customHeight="1">
@@ -3123,19 +3123,19 @@
         <v>46227.0</v>
       </c>
       <c r="E20" s="6" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="F20" s="26" t="s">
         <v>116</v>
       </c>
       <c r="G20" s="12" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="H20" s="6" t="s">
         <v>38</v>
       </c>
       <c r="J20" s="6" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="21" ht="22.5" customHeight="1">
@@ -3152,13 +3152,13 @@
         <v>46227.0</v>
       </c>
       <c r="E21" s="29" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="F21" s="30" t="s">
         <v>118</v>
       </c>
       <c r="G21" s="31" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="H21" s="6" t="s">
         <v>38</v>
@@ -3167,7 +3167,7 @@
         <v>119</v>
       </c>
       <c r="J21" s="33" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="22" ht="22.5" customHeight="1">
@@ -3184,13 +3184,13 @@
         <v>46227.0</v>
       </c>
       <c r="E22" s="6" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="F22" s="7" t="s">
         <v>116</v>
       </c>
       <c r="G22" s="12" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="H22" s="6" t="s">
         <v>38</v>
@@ -3213,19 +3213,19 @@
         <v>46227.0</v>
       </c>
       <c r="E23" s="6" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="F23" s="7" t="s">
         <v>116</v>
       </c>
       <c r="G23" s="12" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="H23" s="6" t="s">
         <v>38</v>
       </c>
       <c r="J23" s="6" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="24" ht="22.5" customHeight="1">
@@ -3242,13 +3242,13 @@
         <v>46227.0</v>
       </c>
       <c r="E24" s="6" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="F24" s="7" t="s">
         <v>116</v>
       </c>
       <c r="G24" s="12" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="H24" s="6" t="s">
         <v>38</v>
@@ -3271,19 +3271,19 @@
         <v>46227.0</v>
       </c>
       <c r="E25" s="6" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="F25" s="7" t="s">
         <v>116</v>
       </c>
       <c r="G25" s="12" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="H25" s="6" t="s">
         <v>38</v>
       </c>
       <c r="J25" s="6" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="26" ht="22.5" customHeight="1">
@@ -3300,13 +3300,13 @@
         <v>46227.0</v>
       </c>
       <c r="E26" s="6" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="F26" s="7" t="s">
         <v>116</v>
       </c>
       <c r="G26" s="12" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="H26" s="6" t="s">
         <v>38</v>
@@ -3329,19 +3329,19 @@
         <v>46227.0</v>
       </c>
       <c r="E27" s="6" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="F27" s="7" t="s">
         <v>116</v>
       </c>
       <c r="G27" s="12" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="H27" s="6" t="s">
         <v>38</v>
       </c>
       <c r="J27" s="6" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="28" ht="22.5" customHeight="1">
@@ -3358,13 +3358,13 @@
         <v>46227.0</v>
       </c>
       <c r="E28" s="6" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="F28" s="7" t="s">
         <v>116</v>
       </c>
       <c r="G28" s="12" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="H28" s="6" t="s">
         <v>38</v>
@@ -3387,19 +3387,19 @@
         <v>46227.0</v>
       </c>
       <c r="E29" s="6" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="F29" s="7" t="s">
         <v>118</v>
       </c>
       <c r="G29" s="12" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="H29" s="6" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="J29" s="6" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="30" ht="22.5" customHeight="1">
@@ -3416,22 +3416,22 @@
         <v>46227.0</v>
       </c>
       <c r="E30" s="6" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="F30" s="7" t="s">
         <v>118</v>
       </c>
       <c r="G30" s="12" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="H30" s="6" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="I30" s="37" t="s">
         <v>119</v>
       </c>
       <c r="J30" s="6" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="31" ht="22.5" customHeight="1">
@@ -3448,16 +3448,16 @@
         <v>46227.0</v>
       </c>
       <c r="E31" s="6" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="F31" s="7" t="s">
         <v>118</v>
       </c>
       <c r="G31" s="12" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="H31" s="6" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="I31" s="6" t="s">
         <v>122</v>
@@ -3477,19 +3477,19 @@
         <v>46227.0</v>
       </c>
       <c r="E32" s="6" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="F32" s="7" t="s">
         <v>118</v>
       </c>
       <c r="G32" s="12" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="H32" s="6" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="J32" s="6" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="33" ht="22.5" customHeight="1">
@@ -3506,22 +3506,22 @@
         <v>46227.0</v>
       </c>
       <c r="E33" s="41" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="F33" s="42" t="s">
         <v>118</v>
       </c>
       <c r="G33" s="43" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="H33" s="41" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="I33" s="44" t="s">
         <v>119</v>
       </c>
       <c r="J33" s="45" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="34" ht="22.5" customHeight="1">
@@ -3538,16 +3538,16 @@
         <v>46227.0</v>
       </c>
       <c r="E34" s="6" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="F34" s="7" t="s">
         <v>118</v>
       </c>
       <c r="G34" s="12" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="H34" s="6" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="I34" s="6" t="s">
         <v>122</v>
@@ -3567,19 +3567,19 @@
         <v>46227.0</v>
       </c>
       <c r="E35" s="6" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="F35" s="7" t="s">
         <v>118</v>
       </c>
       <c r="G35" s="12" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="H35" s="6" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="J35" s="6" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="36" ht="22.5" customHeight="1">
@@ -3596,16 +3596,16 @@
         <v>46227.0</v>
       </c>
       <c r="E36" s="6" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="F36" s="7" t="s">
         <v>118</v>
       </c>
       <c r="G36" s="12" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="H36" s="6" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="I36" s="6" t="s">
         <v>122</v>
@@ -3625,19 +3625,19 @@
         <v>46227.0</v>
       </c>
       <c r="E37" s="6" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="F37" s="7" t="s">
         <v>118</v>
       </c>
       <c r="G37" s="12" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="H37" s="6" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="J37" s="6" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="38" ht="22.5" customHeight="1">
@@ -3654,16 +3654,16 @@
         <v>46227.0</v>
       </c>
       <c r="E38" s="6" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="F38" s="7" t="s">
         <v>118</v>
       </c>
       <c r="G38" s="12" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="H38" s="6" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="I38" s="6" t="s">
         <v>122</v>
@@ -3683,19 +3683,19 @@
         <v>46227.0</v>
       </c>
       <c r="E39" s="6" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="F39" s="7" t="s">
         <v>118</v>
       </c>
       <c r="G39" s="12" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="H39" s="6" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="J39" s="6" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="40" ht="22.5" customHeight="1">
@@ -3712,16 +3712,16 @@
         <v>46227.0</v>
       </c>
       <c r="E40" s="6" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="F40" s="7" t="s">
         <v>118</v>
       </c>
       <c r="G40" s="12" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="H40" s="6" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="I40" s="6" t="s">
         <v>122</v>

</xml_diff>

<commit_message>
Update notebooks folder to include GRCm39 examples
</commit_message>
<xml_diff>
--- a/data/files_provenance_ECCB-2026-T6.xlsx
+++ b/data/files_provenance_ECCB-2026-T6.xlsx
@@ -10,7 +10,7 @@
   <calcPr/>
   <extLst>
     <ext uri="GoogleSheetsCustomDataVersion2">
-      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId6" roundtripDataChecksum="Ugc4rKcaPgtpvzq7RTdx3umEwMpD/wFu9qPvXQvgekY="/>
+      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId6" roundtripDataChecksum="EbTgUhqVE3TwLMvgv8HVAj0/LMrGaoFh36sNlHdV53I="/>
     </ext>
   </extLst>
 </workbook>
@@ -58,70 +58,76 @@
     <t>GRCh38-cCRE-colors18062026.bed.gz</t>
   </si>
   <si>
+    <t>ENCODE</t>
+  </si>
+  <si>
     <t>GRCh38-cCREs.bed</t>
   </si>
   <si>
-    <t>ENCODE</t>
-  </si>
-  <si>
     <t>ENCFF345CWR.atac.bed</t>
   </si>
   <si>
+    <t>ENCFF345CWR.bed</t>
+  </si>
+  <si>
     <t>ENCODE SCREEN</t>
   </si>
   <si>
-    <t>ENCFF345CWR.bed</t>
-  </si>
-  <si>
     <t>https://screen.wenglab.org/downloads</t>
   </si>
   <si>
     <t>https://www.encodeproject.org/experiments/ENCSR903GMO/</t>
   </si>
   <si>
+    <t>ENCODE4 v1.8.0</t>
+  </si>
+  <si>
     <t>V4</t>
   </si>
   <si>
+    <t>mm10</t>
+  </si>
+  <si>
     <t>GRCh38</t>
   </si>
   <si>
+    <t>Rename to include assay type</t>
+  </si>
+  <si>
     <t>Added feature colors. Gzip compression</t>
   </si>
   <si>
-    <t>ENCODE4 v1.8.0</t>
-  </si>
-  <si>
     <t>0-based</t>
   </si>
   <si>
-    <t>mm10</t>
-  </si>
-  <si>
-    <t>Rename to include assay type</t>
+    <t>ENCFF633ETU.atac.chr6.5911252-7710120.bw</t>
+  </si>
+  <si>
+    <t>ENCFF633ETU.bigWig</t>
   </si>
   <si>
     <t>GRCh38-cCRE-colors18062026.bed.idx</t>
   </si>
   <si>
-    <t>ENCFF633ETU.atac.chr6.5911252-7710120.bw</t>
-  </si>
-  <si>
     <t>GRCh38-cCRE-colors18062026.bed</t>
   </si>
   <si>
-    <t>ENCFF633ETU.bigWig</t>
+    <t xml:space="preserve">Rename to include assay type. Trimming </t>
+  </si>
+  <si>
+    <t>ENCFF053ITU.k27ac.bed</t>
+  </si>
+  <si>
+    <t>ENCFF053ITU.bed</t>
+  </si>
+  <si>
+    <t>https://www.encodeproject.org/experiments/ENCSR311YPF/</t>
   </si>
   <si>
     <t>Bed file index</t>
   </si>
   <si>
-    <t xml:space="preserve">Rename to include assay type. Trimming </t>
-  </si>
-  <si>
-    <t>ENCFF053ITU.k27ac.bed</t>
-  </si>
-  <si>
-    <t>ENCFF053ITU.bed</t>
+    <t>ENCODE4 v1.5.1</t>
   </si>
   <si>
     <t>GRCm39-cCRE-colors18062026.bed.gz</t>
@@ -130,7 +136,10 @@
     <t>mm10-cCREs.bed</t>
   </si>
   <si>
-    <t>https://www.encodeproject.org/experiments/ENCSR311YPF/</t>
+    <t>ENCFF607CHT.k27ac.chr6.5911252-7710120.bw</t>
+  </si>
+  <si>
+    <t>ENCFF607CHT.bigWig</t>
   </si>
   <si>
     <t>GRCm39</t>
@@ -139,16 +148,16 @@
     <t>Liftover from mm10, add feature colors. Gzip compression</t>
   </si>
   <si>
+    <t>ENCFF079TUC.k4me3.bed</t>
+  </si>
+  <si>
     <t>mm10-cCRE-colors18062026.bed.gz</t>
   </si>
   <si>
-    <t>ENCODE4 v1.5.1</t>
-  </si>
-  <si>
-    <t>ENCFF607CHT.k27ac.chr6.5911252-7710120.bw</t>
-  </si>
-  <si>
-    <t>ENCFF607CHT.bigWig</t>
+    <t>ENCFF079TUC.bed</t>
+  </si>
+  <si>
+    <t>https://www.encodeproject.org/experiments/ENCSR835BZO/</t>
   </si>
   <si>
     <t>HCT116-cCRE.chr8.bed</t>
@@ -157,13 +166,10 @@
     <t>ENCFF431JDU_ENCFF964OOU_ENCFF787LMI_ENCFF388PVO.bed</t>
   </si>
   <si>
-    <t>ENCFF079TUC.k4me3.bed</t>
-  </si>
-  <si>
-    <t>ENCFF079TUC.bed</t>
-  </si>
-  <si>
-    <t>https://www.encodeproject.org/experiments/ENCSR835BZO/</t>
+    <t>ENCFF798ETE.k4me3.chr6.5911252-7710120.bw</t>
+  </si>
+  <si>
+    <t>ENCFF798ETE.bigWig</t>
   </si>
   <si>
     <t>Filter chr8 features. Rename. Gzip compression.</t>
@@ -172,10 +178,10 @@
     <t>Homo_sapiens.GRCh38.regulatory_features.v116.bb</t>
   </si>
   <si>
-    <t>ENCFF798ETE.k4me3.chr6.5911252-7710120.bw</t>
-  </si>
-  <si>
-    <t>ENCFF798ETE.bigWig</t>
+    <t>ENCFF217ZPW.k4me1.bed</t>
+  </si>
+  <si>
+    <t>ENCFF217ZPW.bed</t>
   </si>
   <si>
     <t>Ensembl Regulation</t>
@@ -184,42 +190,36 @@
     <t>https://regulation.ensembl.org/regulatory_features/homo_sapiens</t>
   </si>
   <si>
-    <t>ENCFF217ZPW.k4me1.bed</t>
-  </si>
-  <si>
-    <t>ENCFF217ZPW.bed</t>
+    <t>https://www.encodeproject.org/experiments/ENCSR496TBX/</t>
   </si>
   <si>
     <t>2025-12</t>
   </si>
   <si>
-    <t>https://www.encodeproject.org/experiments/ENCSR496TBX/</t>
+    <t>ENCODE4 v1.6.1</t>
   </si>
   <si>
     <t>Homo_sapiens.GRCh38.regulatory_features.v116.gff3.gz</t>
   </si>
   <si>
-    <t>ENCODE4 v1.6.1</t>
-  </si>
-  <si>
     <t>ENCFF013ALT.k4me1.chr6.5911252-7710120.bw</t>
   </si>
   <si>
+    <t>ENCFF013ALT.bigWig</t>
+  </si>
+  <si>
     <t>1-based</t>
   </si>
   <si>
-    <t>ENCFF013ALT.bigWig</t>
-  </si>
-  <si>
     <t>Mus_musculus.GRCm39.regulatory_features.v116.bb</t>
   </si>
   <si>
+    <t>ENCFF240LRP.dnase.bed</t>
+  </si>
+  <si>
     <t>https://regulation.ensembl.org/regulatory_features/mus_musculus</t>
   </si>
   <si>
-    <t>ENCFF240LRP.dnase.bed</t>
-  </si>
-  <si>
     <t>ENCFF240LRP.bed</t>
   </si>
   <si>
@@ -238,7 +238,7 @@
     <t>ENCFF906MKW.bigWig</t>
   </si>
   <si>
-    <t>Vista</t>
+    <t>VISTA</t>
   </si>
   <si>
     <t>vistaEnhancers_GRCh38.bb</t>
@@ -247,42 +247,42 @@
     <t>vistaEnhancers.bb</t>
   </si>
   <si>
+    <t>UCSC</t>
+  </si>
+  <si>
+    <t>https://hgdownload.soe.ucsc.edu/gbdb/hg38/vistaEnhancers/</t>
+  </si>
+  <si>
     <t>ENCFF296ZZB.atac.bed</t>
   </si>
   <si>
-    <t>UCSC</t>
-  </si>
-  <si>
     <t>ENCFF296ZZB.bed</t>
   </si>
   <si>
-    <t>https://hgdownload.soe.ucsc.edu/gbdb/hg38/vistaEnhancers/</t>
-  </si>
-  <si>
     <t>https://www.encodeproject.org/experiments/ENCSR872WGW/</t>
   </si>
   <si>
+    <t>01/07/2026</t>
+  </si>
+  <si>
+    <t>Rename</t>
+  </si>
+  <si>
     <t>ENCODE4 v1.9.1</t>
   </si>
   <si>
-    <t>01/07/2026</t>
-  </si>
-  <si>
-    <t>Rename</t>
+    <t>Fantom5</t>
   </si>
   <si>
     <t>ENCFF624HRW.atac.chr8.126229903-128914986.bw</t>
   </si>
   <si>
+    <t>F5.hg38.enhancers.bed.gz</t>
+  </si>
+  <si>
     <t>ENCFF624HRW.bw</t>
   </si>
   <si>
-    <t>Fantom5</t>
-  </si>
-  <si>
-    <t>F5.hg38.enhancers.bed.gz</t>
-  </si>
-  <si>
     <t>F5.hg38.enhancers.bed</t>
   </si>
   <si>
@@ -292,43 +292,43 @@
     <t>https://fantom.gsc.riken.jp/5/datafiles/reprocessed/hg38_v9/extra/enhancer/</t>
   </si>
   <si>
+    <t>V9</t>
+  </si>
+  <si>
     <t>ENCFF711MPL.k4me3.bed</t>
   </si>
   <si>
     <t>ENCFF711MPL.bed</t>
   </si>
   <si>
-    <t>V9</t>
+    <t>Gzip compression.</t>
   </si>
   <si>
     <t>https://www.encodeproject.org/experiments/ENCSR333OPW/</t>
   </si>
   <si>
-    <t>Gzip compression.</t>
-  </si>
-  <si>
     <t>RefSeq</t>
   </si>
   <si>
+    <t>GCF_000001405.40_GRCh38.p14_genomic.RefSeqFE.gff.gz</t>
+  </si>
+  <si>
+    <t>GCF_000001405.40_GRCh38.p14_genomic.gff</t>
+  </si>
+  <si>
     <t xml:space="preserve">ENCODE4 v1.5.1 </t>
   </si>
   <si>
-    <t>GCF_000001405.40_GRCh38.p14_genomic.RefSeqFE.gff.gz</t>
-  </si>
-  <si>
-    <t>GCF_000001405.40_GRCh38.p14_genomic.gff</t>
-  </si>
-  <si>
     <t>https://ftp.ncbi.nlm.nih.gov/genomes/refseq/vertebrate_mammalian/Homo_sapiens/latest_assembly_versions/GCF_000001405.40_GRCh38.p14/</t>
   </si>
   <si>
     <t>ENCFF394IMO.k4me3.chr8.126229903-128914986.bw</t>
   </si>
   <si>
+    <t>08/01/2025</t>
+  </si>
+  <si>
     <t>ENCFF394IMO.bw</t>
-  </si>
-  <si>
-    <t>08/01/2025</t>
   </si>
   <si>
     <t>Extract RefSeqFE annotations, rename chromosome, remove biological_region features. Gzip compression.</t>
@@ -842,7 +842,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:J13" displayName="Table2" name="Table2" id="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:J13" displayName="Table2" name="Table2" id="2">
   <tableColumns count="10">
     <tableColumn name="Folder" id="1"/>
     <tableColumn name="File name" id="2"/>
@@ -860,7 +860,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:J40" displayName="Table1" name="Table1" id="2">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:J40" displayName="Table1" name="Table1" id="1">
   <tableColumns count="10">
     <tableColumn name="Folder" id="1"/>
     <tableColumn name="File name" id="2"/>
@@ -1130,150 +1130,150 @@
         <v>12</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D2" s="5">
         <v>46191.0</v>
       </c>
       <c r="E2" s="6" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F2" s="7" t="s">
         <v>18</v>
       </c>
       <c r="G2" s="8" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="H2" s="6" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="I2" s="9" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="J2" s="6" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
     </row>
     <row r="3" ht="22.5" customHeight="1">
       <c r="A3" s="2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D3" s="5"/>
       <c r="E3" s="6" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F3" s="10"/>
       <c r="G3" s="8" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="H3" s="9" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="I3" s="9" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="J3" s="6"/>
     </row>
     <row r="4" ht="22.5" customHeight="1">
       <c r="A4" s="11" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="D4" s="5">
         <v>46191.0</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F4" s="7" t="s">
         <v>18</v>
       </c>
       <c r="G4" s="8" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="H4" s="6" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="I4" s="9" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="J4" s="6" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
     </row>
     <row r="5" ht="22.5" customHeight="1">
       <c r="A5" s="11" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="D5" s="5">
         <v>46191.0</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F5" s="7" t="s">
         <v>18</v>
       </c>
       <c r="G5" s="8" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="H5" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="I5" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="I5" s="9" t="s">
-        <v>22</v>
-      </c>
       <c r="J5" s="6" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
     </row>
     <row r="6" ht="22.5" customHeight="1">
       <c r="A6" s="11" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="D6" s="5">
         <v>46227.0</v>
       </c>
       <c r="E6" s="6" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F6" s="7" t="s">
         <v>18</v>
       </c>
       <c r="G6" s="8" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="H6" s="6" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="I6" s="9" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="J6" s="6" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
     </row>
     <row r="7" ht="22.5" customHeight="1">
@@ -1281,28 +1281,28 @@
         <v>11</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="D7" s="5">
         <v>46206.0</v>
       </c>
       <c r="E7" s="6" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="F7" s="7" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="G7" s="12" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="H7" s="6" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="J7" s="6" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
     </row>
     <row r="8" ht="22.5" customHeight="1">
@@ -1310,28 +1310,28 @@
         <v>11</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="D8" s="5">
         <v>46191.0</v>
       </c>
       <c r="E8" s="6" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="F8" s="7" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="G8" s="12" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="H8" s="6" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="J8" s="6" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
     </row>
     <row r="9" ht="22.5" customHeight="1">
@@ -1348,19 +1348,19 @@
         <v>46206.0</v>
       </c>
       <c r="E9" s="6" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="F9" s="13" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="G9" s="12" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="H9" s="6" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="J9" s="6" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
     </row>
     <row r="10" ht="22.5" customHeight="1">
@@ -1377,19 +1377,19 @@
         <v>46191.0</v>
       </c>
       <c r="E10" s="6" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="F10" s="13" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="G10" s="12" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="H10" s="6" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="J10" s="6" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
     </row>
     <row r="11" ht="15.75" customHeight="1">
@@ -1406,30 +1406,30 @@
         <v>46251.0</v>
       </c>
       <c r="E11" s="18" t="s">
+        <v>76</v>
+      </c>
+      <c r="F11" s="19" t="s">
         <v>77</v>
       </c>
-      <c r="F11" s="19" t="s">
-        <v>79</v>
-      </c>
       <c r="G11" s="20" t="s">
+        <v>81</v>
+      </c>
+      <c r="H11" s="21" t="s">
+        <v>23</v>
+      </c>
+      <c r="I11" s="22" t="s">
         <v>82</v>
       </c>
-      <c r="H11" s="21" t="s">
-        <v>21</v>
-      </c>
-      <c r="I11" s="22" t="s">
-        <v>83</v>
-      </c>
       <c r="J11" s="6" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
     </row>
     <row r="12" ht="15.75" customHeight="1">
       <c r="A12" s="14" t="s">
+        <v>84</v>
+      </c>
+      <c r="B12" s="23" t="s">
         <v>86</v>
-      </c>
-      <c r="B12" s="23" t="s">
-        <v>87</v>
       </c>
       <c r="C12" s="23" t="s">
         <v>88</v>
@@ -1444,16 +1444,16 @@
         <v>90</v>
       </c>
       <c r="G12" s="24" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="H12" s="21" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="I12" s="23" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="J12" s="6" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
     </row>
     <row r="13" ht="15.75" customHeight="1">
@@ -1461,10 +1461,10 @@
         <v>96</v>
       </c>
       <c r="B13" s="23" t="s">
+        <v>97</v>
+      </c>
+      <c r="C13" s="23" t="s">
         <v>98</v>
-      </c>
-      <c r="C13" s="23" t="s">
-        <v>99</v>
       </c>
       <c r="D13" s="17">
         <v>46251.0</v>
@@ -1476,16 +1476,16 @@
         <v>100</v>
       </c>
       <c r="G13" s="20" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="H13" s="21" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="I13" s="22" t="s">
         <v>104</v>
       </c>
       <c r="J13" s="21" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
     </row>
     <row r="14" ht="15.75" customHeight="1"/>
@@ -2562,254 +2562,254 @@
     </row>
     <row r="2" ht="22.5" customHeight="1">
       <c r="A2" s="4" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B2" s="4" t="s">
         <v>15</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D2" s="5">
         <v>46226.0</v>
       </c>
       <c r="E2" s="6" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="F2" s="7" t="s">
         <v>19</v>
       </c>
       <c r="G2" s="6" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="H2" s="6" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="I2" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="J2" s="6" t="s">
         <v>26</v>
-      </c>
-      <c r="J2" s="6" t="s">
-        <v>24</v>
       </c>
     </row>
     <row r="3" ht="22.5" customHeight="1">
       <c r="A3" s="4" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B3" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="C3" s="4" t="s">
         <v>28</v>
-      </c>
-      <c r="C3" s="4" t="s">
-        <v>30</v>
       </c>
       <c r="D3" s="5">
         <v>46226.0</v>
       </c>
       <c r="E3" s="6" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="F3" s="7" t="s">
         <v>19</v>
       </c>
       <c r="G3" s="6" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="H3" s="6" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="I3" s="6" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="4" ht="22.5" customHeight="1">
       <c r="A4" s="4" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B4" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="C4" s="4" t="s">
         <v>33</v>
-      </c>
-      <c r="C4" s="4" t="s">
-        <v>34</v>
       </c>
       <c r="D4" s="5">
         <v>46226.0</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="F4" s="7" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="G4" s="6" t="s">
-        <v>41</v>
+        <v>36</v>
       </c>
       <c r="H4" s="6" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="I4" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="J4" s="6" t="s">
         <v>26</v>
-      </c>
-      <c r="J4" s="6" t="s">
-        <v>24</v>
       </c>
     </row>
     <row r="5" ht="22.5" customHeight="1">
       <c r="A5" s="4" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="D5" s="5">
         <v>46226.0</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="F5" s="7" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="G5" s="6" t="s">
-        <v>41</v>
+        <v>36</v>
       </c>
       <c r="H5" s="6" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="I5" s="6" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="6" ht="22.5" customHeight="1">
       <c r="A6" s="4" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="D6" s="5">
         <v>46226.0</v>
       </c>
       <c r="E6" s="6" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="F6" s="7" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="G6" s="6" t="s">
-        <v>41</v>
+        <v>36</v>
       </c>
       <c r="H6" s="6" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="I6" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="J6" s="6" t="s">
         <v>26</v>
-      </c>
-      <c r="J6" s="6" t="s">
-        <v>24</v>
       </c>
     </row>
     <row r="7" ht="22.5" customHeight="1">
       <c r="A7" s="4" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="D7" s="5">
         <v>46226.0</v>
       </c>
       <c r="E7" s="6" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="F7" s="7" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="G7" s="6" t="s">
-        <v>41</v>
+        <v>36</v>
       </c>
       <c r="H7" s="6" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="I7" s="6" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="8" ht="22.5" customHeight="1">
       <c r="A8" s="4" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="D8" s="5">
         <v>46226.0</v>
       </c>
       <c r="E8" s="6" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="F8" s="7" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="G8" s="6" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="H8" s="6" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="I8" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="J8" s="6" t="s">
         <v>26</v>
-      </c>
-      <c r="J8" s="6" t="s">
-        <v>24</v>
       </c>
     </row>
     <row r="9" ht="22.5" customHeight="1">
       <c r="A9" s="4" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B9" s="4" t="s">
         <v>61</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="D9" s="5">
         <v>46226.0</v>
       </c>
       <c r="E9" s="6" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="F9" s="7" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="G9" s="6" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="H9" s="6" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="I9" s="6" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="10" ht="22.5" customHeight="1">
       <c r="A10" s="4" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="C10" s="4" t="s">
         <v>67</v>
@@ -2818,7 +2818,7 @@
         <v>46162.0</v>
       </c>
       <c r="E10" s="6" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="F10" s="7" t="s">
         <v>68</v>
@@ -2827,18 +2827,18 @@
         <v>69</v>
       </c>
       <c r="H10" s="6" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="I10" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="J10" s="6" t="s">
         <v>26</v>
-      </c>
-      <c r="J10" s="6" t="s">
-        <v>24</v>
       </c>
     </row>
     <row r="11" ht="22.5" customHeight="1">
       <c r="A11" s="4" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B11" s="4" t="s">
         <v>71</v>
@@ -2850,7 +2850,7 @@
         <v>46162.0</v>
       </c>
       <c r="E11" s="6" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="F11" s="7" t="s">
         <v>68</v>
@@ -2859,137 +2859,137 @@
         <v>69</v>
       </c>
       <c r="H11" s="6" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="I11" s="6" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="12" ht="22.5" customHeight="1">
       <c r="A12" s="4" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="D12" s="5">
         <v>46162.0</v>
       </c>
       <c r="E12" s="6" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="F12" s="7" t="s">
         <v>80</v>
       </c>
       <c r="G12" s="6" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="H12" s="6" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="I12" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="J12" s="6" t="s">
         <v>26</v>
-      </c>
-      <c r="J12" s="6" t="s">
-        <v>24</v>
       </c>
     </row>
     <row r="13" ht="22.5" customHeight="1">
       <c r="A13" s="4" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="D13" s="5">
         <v>46162.0</v>
       </c>
       <c r="E13" s="6" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="F13" s="7" t="s">
         <v>80</v>
       </c>
       <c r="G13" s="6" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="H13" s="6" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="I13" s="6" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="14" ht="22.5" customHeight="1">
       <c r="A14" s="4" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="D14" s="5">
         <v>46162.0</v>
       </c>
       <c r="E14" s="6" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="F14" s="7" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="G14" s="6" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="H14" s="6" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="I14" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="J14" s="6" t="s">
         <v>26</v>
-      </c>
-      <c r="J14" s="6" t="s">
-        <v>24</v>
       </c>
     </row>
     <row r="15" ht="22.5" customHeight="1">
       <c r="A15" s="4" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B15" s="4" t="s">
         <v>101</v>
       </c>
       <c r="C15" s="6" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="D15" s="5">
         <v>46162.0</v>
       </c>
       <c r="E15" s="6" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="F15" s="7" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="G15" s="6" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="H15" s="6" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="I15" s="6" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="16" ht="22.5" customHeight="1">
       <c r="A16" s="4" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B16" s="4" t="s">
         <v>105</v>
@@ -3001,27 +3001,27 @@
         <v>46162.0</v>
       </c>
       <c r="E16" s="6" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="F16" s="7" t="s">
         <v>107</v>
       </c>
       <c r="G16" s="6" t="s">
-        <v>41</v>
+        <v>36</v>
       </c>
       <c r="H16" s="6" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="I16" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="J16" s="6" t="s">
         <v>26</v>
-      </c>
-      <c r="J16" s="6" t="s">
-        <v>24</v>
       </c>
     </row>
     <row r="17" ht="22.5" customHeight="1">
       <c r="A17" s="4" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B17" s="4" t="s">
         <v>108</v>
@@ -3033,24 +3033,24 @@
         <v>46162.0</v>
       </c>
       <c r="E17" s="6" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="F17" s="7" t="s">
         <v>107</v>
       </c>
       <c r="G17" s="6" t="s">
-        <v>41</v>
+        <v>36</v>
       </c>
       <c r="H17" s="6" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="I17" s="6" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="18" ht="22.5" customHeight="1">
       <c r="A18" s="4" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B18" s="4" t="s">
         <v>110</v>
@@ -3062,27 +3062,27 @@
         <v>46162.0</v>
       </c>
       <c r="E18" s="6" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="F18" s="7" t="s">
         <v>112</v>
       </c>
       <c r="G18" s="6" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="H18" s="6" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="I18" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="J18" s="6" t="s">
         <v>26</v>
-      </c>
-      <c r="J18" s="6" t="s">
-        <v>24</v>
       </c>
     </row>
     <row r="19" ht="22.5" customHeight="1">
       <c r="A19" s="4" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B19" s="4" t="s">
         <v>113</v>
@@ -3094,19 +3094,19 @@
         <v>46162.0</v>
       </c>
       <c r="E19" s="6" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="F19" s="7" t="s">
         <v>112</v>
       </c>
       <c r="G19" s="6" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="H19" s="6" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="I19" s="6" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="20" ht="22.5" customHeight="1">
@@ -3123,19 +3123,19 @@
         <v>46227.0</v>
       </c>
       <c r="E20" s="6" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="F20" s="26" t="s">
         <v>116</v>
       </c>
       <c r="G20" s="12" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="H20" s="6" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="J20" s="6" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
     </row>
     <row r="21" ht="22.5" customHeight="1">
@@ -3152,22 +3152,22 @@
         <v>46227.0</v>
       </c>
       <c r="E21" s="29" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="F21" s="30" t="s">
         <v>118</v>
       </c>
       <c r="G21" s="31" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="H21" s="6" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="I21" s="32" t="s">
         <v>119</v>
       </c>
       <c r="J21" s="33" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
     </row>
     <row r="22" ht="22.5" customHeight="1">
@@ -3184,16 +3184,16 @@
         <v>46227.0</v>
       </c>
       <c r="E22" s="6" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="F22" s="7" t="s">
         <v>116</v>
       </c>
       <c r="G22" s="12" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="H22" s="6" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="I22" s="6" t="s">
         <v>122</v>
@@ -3213,19 +3213,19 @@
         <v>46227.0</v>
       </c>
       <c r="E23" s="6" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="F23" s="7" t="s">
         <v>116</v>
       </c>
       <c r="G23" s="12" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="H23" s="6" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="J23" s="6" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
     </row>
     <row r="24" ht="22.5" customHeight="1">
@@ -3242,16 +3242,16 @@
         <v>46227.0</v>
       </c>
       <c r="E24" s="6" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="F24" s="7" t="s">
         <v>116</v>
       </c>
       <c r="G24" s="12" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="H24" s="6" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="I24" s="6" t="s">
         <v>122</v>
@@ -3271,19 +3271,19 @@
         <v>46227.0</v>
       </c>
       <c r="E25" s="6" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="F25" s="7" t="s">
         <v>116</v>
       </c>
       <c r="G25" s="12" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="H25" s="6" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="J25" s="6" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
     </row>
     <row r="26" ht="22.5" customHeight="1">
@@ -3300,16 +3300,16 @@
         <v>46227.0</v>
       </c>
       <c r="E26" s="6" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="F26" s="7" t="s">
         <v>116</v>
       </c>
       <c r="G26" s="12" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="H26" s="6" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="I26" s="6" t="s">
         <v>122</v>
@@ -3329,19 +3329,19 @@
         <v>46227.0</v>
       </c>
       <c r="E27" s="6" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="F27" s="7" t="s">
         <v>116</v>
       </c>
       <c r="G27" s="12" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="H27" s="6" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="J27" s="6" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
     </row>
     <row r="28" ht="22.5" customHeight="1">
@@ -3358,16 +3358,16 @@
         <v>46227.0</v>
       </c>
       <c r="E28" s="6" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="F28" s="7" t="s">
         <v>116</v>
       </c>
       <c r="G28" s="12" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="H28" s="6" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="I28" s="6" t="s">
         <v>122</v>
@@ -3387,19 +3387,19 @@
         <v>46227.0</v>
       </c>
       <c r="E29" s="6" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="F29" s="7" t="s">
         <v>118</v>
       </c>
       <c r="G29" s="12" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="H29" s="6" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="J29" s="6" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
     </row>
     <row r="30" ht="22.5" customHeight="1">
@@ -3416,22 +3416,22 @@
         <v>46227.0</v>
       </c>
       <c r="E30" s="6" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="F30" s="7" t="s">
         <v>118</v>
       </c>
       <c r="G30" s="12" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="H30" s="6" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="I30" s="37" t="s">
         <v>119</v>
       </c>
       <c r="J30" s="6" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
     </row>
     <row r="31" ht="22.5" customHeight="1">
@@ -3448,16 +3448,16 @@
         <v>46227.0</v>
       </c>
       <c r="E31" s="6" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="F31" s="7" t="s">
         <v>118</v>
       </c>
       <c r="G31" s="12" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="H31" s="6" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="I31" s="6" t="s">
         <v>122</v>
@@ -3477,19 +3477,19 @@
         <v>46227.0</v>
       </c>
       <c r="E32" s="6" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="F32" s="7" t="s">
         <v>118</v>
       </c>
       <c r="G32" s="12" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="H32" s="6" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="J32" s="6" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
     </row>
     <row r="33" ht="22.5" customHeight="1">
@@ -3506,22 +3506,22 @@
         <v>46227.0</v>
       </c>
       <c r="E33" s="41" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="F33" s="42" t="s">
         <v>118</v>
       </c>
       <c r="G33" s="43" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="H33" s="41" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="I33" s="44" t="s">
         <v>119</v>
       </c>
       <c r="J33" s="45" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
     </row>
     <row r="34" ht="22.5" customHeight="1">
@@ -3538,16 +3538,16 @@
         <v>46227.0</v>
       </c>
       <c r="E34" s="6" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="F34" s="7" t="s">
         <v>118</v>
       </c>
       <c r="G34" s="12" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="H34" s="6" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="I34" s="6" t="s">
         <v>122</v>
@@ -3567,19 +3567,19 @@
         <v>46227.0</v>
       </c>
       <c r="E35" s="6" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="F35" s="7" t="s">
         <v>118</v>
       </c>
       <c r="G35" s="12" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="H35" s="6" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="J35" s="6" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
     </row>
     <row r="36" ht="22.5" customHeight="1">
@@ -3596,16 +3596,16 @@
         <v>46227.0</v>
       </c>
       <c r="E36" s="6" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="F36" s="7" t="s">
         <v>118</v>
       </c>
       <c r="G36" s="12" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="H36" s="6" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="I36" s="6" t="s">
         <v>122</v>
@@ -3625,19 +3625,19 @@
         <v>46227.0</v>
       </c>
       <c r="E37" s="6" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="F37" s="7" t="s">
         <v>118</v>
       </c>
       <c r="G37" s="12" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="H37" s="6" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="J37" s="6" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
     </row>
     <row r="38" ht="22.5" customHeight="1">
@@ -3654,16 +3654,16 @@
         <v>46227.0</v>
       </c>
       <c r="E38" s="6" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="F38" s="7" t="s">
         <v>118</v>
       </c>
       <c r="G38" s="12" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="H38" s="6" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="I38" s="6" t="s">
         <v>122</v>
@@ -3683,19 +3683,19 @@
         <v>46227.0</v>
       </c>
       <c r="E39" s="6" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="F39" s="7" t="s">
         <v>118</v>
       </c>
       <c r="G39" s="12" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="H39" s="6" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="J39" s="6" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
     </row>
     <row r="40" ht="22.5" customHeight="1">
@@ -3712,16 +3712,16 @@
         <v>46227.0</v>
       </c>
       <c r="E40" s="6" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="F40" s="7" t="s">
         <v>118</v>
       </c>
       <c r="G40" s="12" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="H40" s="6" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="I40" s="6" t="s">
         <v>122</v>

</xml_diff>